<commit_message>
add code for formulary and brochure document search and validate
</commit_message>
<xml_diff>
--- a/data/marketplace/MarketplacePlansData.xlsx
+++ b/data/marketplace/MarketplacePlansData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://molinahealthcare-my.sharepoint.com/personal/naresh_jangid_molinahealthcare_com/Documents/Automation/molina_automation/marketplace/data/marketplace/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="11_E9EF72481E37605E54A31C6A4016A4F540A16DA8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C18B1B3-D99B-4BDB-B0C9-7211EF459C6E}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="11_E9EF72481E37605E54A31C6A4016A4F540A16DA8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D5B12C28-2B7A-4425-83F7-2FE53783087F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5417,9 +5417,9 @@
         <v>260</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>357</v>
+        <v>9</v>
       </c>
       <c r="B89" t="s">
         <v>261</v>
@@ -6751,7 +6751,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>9</v>
       </c>
@@ -10057,9 +10057,9 @@
         <v>675</v>
       </c>
     </row>
-    <row r="249" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B249" t="s">
         <v>676</v>
@@ -10086,9 +10086,9 @@
         <v>679</v>
       </c>
     </row>
-    <row r="250" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B250" t="s">
         <v>680</v>
@@ -10115,9 +10115,9 @@
         <v>681</v>
       </c>
     </row>
-    <row r="251" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B251" t="s">
         <v>682</v>
@@ -10144,9 +10144,9 @@
         <v>683</v>
       </c>
     </row>
-    <row r="252" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B252" t="s">
         <v>684</v>
@@ -10173,9 +10173,9 @@
         <v>685</v>
       </c>
     </row>
-    <row r="253" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B253" t="s">
         <v>686</v>
@@ -10202,9 +10202,9 @@
         <v>687</v>
       </c>
     </row>
-    <row r="254" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B254" t="s">
         <v>688</v>
@@ -10231,9 +10231,9 @@
         <v>689</v>
       </c>
     </row>
-    <row r="255" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B255" t="s">
         <v>690</v>
@@ -10260,9 +10260,9 @@
         <v>691</v>
       </c>
     </row>
-    <row r="256" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B256" t="s">
         <v>692</v>
@@ -10289,9 +10289,9 @@
         <v>693</v>
       </c>
     </row>
-    <row r="257" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B257" t="s">
         <v>694</v>
@@ -10318,9 +10318,9 @@
         <v>695</v>
       </c>
     </row>
-    <row r="258" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B258" t="s">
         <v>696</v>
@@ -10347,9 +10347,9 @@
         <v>697</v>
       </c>
     </row>
-    <row r="259" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B259" t="s">
         <v>698</v>
@@ -10376,9 +10376,9 @@
         <v>699</v>
       </c>
     </row>
-    <row r="260" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B260" t="s">
         <v>700</v>
@@ -10405,9 +10405,9 @@
         <v>701</v>
       </c>
     </row>
-    <row r="261" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B261" t="s">
         <v>702</v>
@@ -10434,9 +10434,9 @@
         <v>703</v>
       </c>
     </row>
-    <row r="262" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B262" t="s">
         <v>704</v>
@@ -10463,9 +10463,9 @@
         <v>705</v>
       </c>
     </row>
-    <row r="263" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B263" t="s">
         <v>706</v>
@@ -10492,9 +10492,9 @@
         <v>707</v>
       </c>
     </row>
-    <row r="264" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B264" t="s">
         <v>708</v>
@@ -10521,9 +10521,9 @@
         <v>709</v>
       </c>
     </row>
-    <row r="265" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B265" t="s">
         <v>710</v>
@@ -10550,9 +10550,9 @@
         <v>712</v>
       </c>
     </row>
-    <row r="266" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B266" t="s">
         <v>713</v>
@@ -10579,9 +10579,9 @@
         <v>714</v>
       </c>
     </row>
-    <row r="267" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B267" t="s">
         <v>715</v>
@@ -10608,9 +10608,9 @@
         <v>717</v>
       </c>
     </row>
-    <row r="268" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B268" t="s">
         <v>718</v>
@@ -10637,9 +10637,9 @@
         <v>719</v>
       </c>
     </row>
-    <row r="269" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B269" t="s">
         <v>720</v>
@@ -10666,9 +10666,9 @@
         <v>721</v>
       </c>
     </row>
-    <row r="270" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A270" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B270" t="s">
         <v>722</v>
@@ -10695,9 +10695,9 @@
         <v>723</v>
       </c>
     </row>
-    <row r="271" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B271" t="s">
         <v>724</v>
@@ -10724,9 +10724,9 @@
         <v>725</v>
       </c>
     </row>
-    <row r="272" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A272" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B272" t="s">
         <v>726</v>
@@ -10753,9 +10753,9 @@
         <v>727</v>
       </c>
     </row>
-    <row r="273" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B273" t="s">
         <v>728</v>
@@ -10782,9 +10782,9 @@
         <v>729</v>
       </c>
     </row>
-    <row r="274" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B274" t="s">
         <v>730</v>
@@ -10811,9 +10811,9 @@
         <v>731</v>
       </c>
     </row>
-    <row r="275" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B275" t="s">
         <v>732</v>
@@ -10840,9 +10840,9 @@
         <v>733</v>
       </c>
     </row>
-    <row r="276" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A276" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B276" t="s">
         <v>734</v>
@@ -10869,9 +10869,9 @@
         <v>735</v>
       </c>
     </row>
-    <row r="277" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A277" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B277" t="s">
         <v>736</v>
@@ -10898,9 +10898,9 @@
         <v>737</v>
       </c>
     </row>
-    <row r="278" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B278" t="s">
         <v>738</v>
@@ -10927,9 +10927,9 @@
         <v>739</v>
       </c>
     </row>
-    <row r="279" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B279" t="s">
         <v>740</v>
@@ -10956,9 +10956,9 @@
         <v>741</v>
       </c>
     </row>
-    <row r="280" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B280" t="s">
         <v>742</v>
@@ -10985,9 +10985,9 @@
         <v>743</v>
       </c>
     </row>
-    <row r="281" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B281" t="s">
         <v>744</v>
@@ -11014,9 +11014,9 @@
         <v>745</v>
       </c>
     </row>
-    <row r="282" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B282" t="s">
         <v>746</v>
@@ -11043,9 +11043,9 @@
         <v>748</v>
       </c>
     </row>
-    <row r="283" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B283" t="s">
         <v>749</v>
@@ -11072,9 +11072,9 @@
         <v>751</v>
       </c>
     </row>
-    <row r="284" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B284" t="s">
         <v>752</v>
@@ -11101,9 +11101,9 @@
         <v>754</v>
       </c>
     </row>
-    <row r="285" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B285" t="s">
         <v>755</v>
@@ -11130,9 +11130,9 @@
         <v>756</v>
       </c>
     </row>
-    <row r="286" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B286" t="s">
         <v>757</v>
@@ -11159,9 +11159,9 @@
         <v>758</v>
       </c>
     </row>
-    <row r="287" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B287" t="s">
         <v>759</v>
@@ -11188,9 +11188,9 @@
         <v>760</v>
       </c>
     </row>
-    <row r="288" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B288" t="s">
         <v>761</v>
@@ -11217,9 +11217,9 @@
         <v>762</v>
       </c>
     </row>
-    <row r="289" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B289" t="s">
         <v>763</v>
@@ -11246,9 +11246,9 @@
         <v>764</v>
       </c>
     </row>
-    <row r="290" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A290" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B290" t="s">
         <v>765</v>
@@ -11275,9 +11275,9 @@
         <v>766</v>
       </c>
     </row>
-    <row r="291" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B291" t="s">
         <v>767</v>
@@ -11304,9 +11304,9 @@
         <v>768</v>
       </c>
     </row>
-    <row r="292" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A292" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B292" t="s">
         <v>769</v>
@@ -11333,9 +11333,9 @@
         <v>770</v>
       </c>
     </row>
-    <row r="293" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A293" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B293" t="s">
         <v>771</v>
@@ -11362,9 +11362,9 @@
         <v>772</v>
       </c>
     </row>
-    <row r="294" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A294" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B294" t="s">
         <v>773</v>
@@ -11391,9 +11391,9 @@
         <v>774</v>
       </c>
     </row>
-    <row r="295" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A295" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B295" t="s">
         <v>775</v>
@@ -11420,9 +11420,9 @@
         <v>777</v>
       </c>
     </row>
-    <row r="296" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B296" t="s">
         <v>778</v>
@@ -11449,9 +11449,9 @@
         <v>779</v>
       </c>
     </row>
-    <row r="297" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A297" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B297" t="s">
         <v>780</v>
@@ -11478,9 +11478,9 @@
         <v>781</v>
       </c>
     </row>
-    <row r="298" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B298" t="s">
         <v>782</v>
@@ -11507,9 +11507,9 @@
         <v>783</v>
       </c>
     </row>
-    <row r="299" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B299" t="s">
         <v>784</v>
@@ -11536,9 +11536,9 @@
         <v>785</v>
       </c>
     </row>
-    <row r="300" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A300" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B300" t="s">
         <v>786</v>
@@ -11565,9 +11565,9 @@
         <v>787</v>
       </c>
     </row>
-    <row r="301" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B301" t="s">
         <v>788</v>
@@ -11594,9 +11594,9 @@
         <v>789</v>
       </c>
     </row>
-    <row r="302" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B302" t="s">
         <v>790</v>
@@ -11623,9 +11623,9 @@
         <v>791</v>
       </c>
     </row>
-    <row r="303" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B303" t="s">
         <v>792</v>
@@ -11652,9 +11652,9 @@
         <v>793</v>
       </c>
     </row>
-    <row r="304" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B304" t="s">
         <v>794</v>
@@ -11681,9 +11681,9 @@
         <v>795</v>
       </c>
     </row>
-    <row r="305" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B305" t="s">
         <v>796</v>
@@ -11710,9 +11710,9 @@
         <v>797</v>
       </c>
     </row>
-    <row r="306" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="B306" t="s">
         <v>798</v>
@@ -12002,15 +12002,15 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:I315" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="0">
+    <filterColumn colId="2">
       <filters>
-        <filter val="Y"/>
+        <filter val="TX"/>
       </filters>
     </filterColumn>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:I88 A90:I134 B89:I89 A136:I315 B135:I135" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:I88 A122:I134 B89:I89 A179:I248 B135:I135 B90:I121 B136:I149 B150:I150 B151:I178 B308:I315 B307:I307 B250:I306 B249:I249" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Updated url in sheet
</commit_message>
<xml_diff>
--- a/data/marketplace/MarketplacePlansData.xlsx
+++ b/data/marketplace/MarketplacePlansData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://molinahealthcare-my.sharepoint.com/personal/naresh_jangid_molinahealthcare_com/Documents/Automation/molina_automation/marketplace/data/marketplace/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_70CE30217927462588B21A62D89D467537775006" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE66B700-B1A6-4FED-8420-B8CC9166D3D8}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="11_70CE30217927462588B21A62D89D467537775006" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B15F36B0-41C2-4005-9C8F-EE767325F417}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Settings" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Plans!A1:I315</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Plans!$A$1:$I$315</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
@@ -2875,13 +2875,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:I315"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="6" max="6" width="11.296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.09765625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="70.3984375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="241.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2910,7 +2914,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2939,7 +2943,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2968,7 +2972,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2997,7 +3001,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3026,7 +3030,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3055,7 +3059,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3084,7 +3088,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -3113,7 +3117,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -3142,7 +3146,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -3171,7 +3175,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -3200,7 +3204,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -3229,7 +3233,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -3258,7 +3262,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -3287,7 +3291,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -3316,7 +3320,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>9</v>
       </c>
@@ -3345,7 +3349,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>9</v>
       </c>
@@ -3374,7 +3378,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>9</v>
       </c>
@@ -3403,7 +3407,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>9</v>
       </c>
@@ -3432,7 +3436,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>9</v>
       </c>
@@ -3461,7 +3465,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>9</v>
       </c>
@@ -3490,7 +3494,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>9</v>
       </c>
@@ -3519,7 +3523,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>9</v>
       </c>
@@ -3548,7 +3552,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>9</v>
       </c>
@@ -3577,7 +3581,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>9</v>
       </c>
@@ -3606,7 +3610,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>9</v>
       </c>
@@ -3635,7 +3639,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>9</v>
       </c>
@@ -3664,7 +3668,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>9</v>
       </c>
@@ -3693,7 +3697,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>9</v>
       </c>
@@ -3722,7 +3726,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>9</v>
       </c>
@@ -3751,7 +3755,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>9</v>
       </c>
@@ -3780,7 +3784,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>9</v>
       </c>
@@ -3809,7 +3813,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>9</v>
       </c>
@@ -3838,7 +3842,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>9</v>
       </c>
@@ -3867,7 +3871,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>9</v>
       </c>
@@ -3896,7 +3900,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>9</v>
       </c>
@@ -3925,7 +3929,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>9</v>
       </c>
@@ -3954,7 +3958,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>9</v>
       </c>
@@ -3983,7 +3987,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>9</v>
       </c>
@@ -4012,7 +4016,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>9</v>
       </c>
@@ -4041,7 +4045,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>9</v>
       </c>
@@ -4070,7 +4074,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>9</v>
       </c>
@@ -4099,7 +4103,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>9</v>
       </c>
@@ -4128,7 +4132,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>9</v>
       </c>
@@ -4157,7 +4161,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>9</v>
       </c>
@@ -4186,7 +4190,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>9</v>
       </c>
@@ -4215,7 +4219,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>9</v>
       </c>
@@ -4244,7 +4248,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>9</v>
       </c>
@@ -4273,7 +4277,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="49" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>9</v>
       </c>
@@ -4302,7 +4306,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="50" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>9</v>
       </c>
@@ -4331,7 +4335,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="51" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>9</v>
       </c>
@@ -4360,7 +4364,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="52" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>9</v>
       </c>
@@ -4389,7 +4393,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="53" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>9</v>
       </c>
@@ -4418,7 +4422,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="54" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>9</v>
       </c>
@@ -4447,7 +4451,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="55" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>9</v>
       </c>
@@ -4476,7 +4480,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="56" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>9</v>
       </c>
@@ -4505,7 +4509,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="57" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>9</v>
       </c>
@@ -4534,7 +4538,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="58" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>9</v>
       </c>
@@ -4563,7 +4567,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="59" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>9</v>
       </c>
@@ -4592,7 +4596,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="60" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>9</v>
       </c>
@@ -4621,7 +4625,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="61" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>9</v>
       </c>
@@ -4650,7 +4654,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="62" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>9</v>
       </c>
@@ -4679,7 +4683,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="63" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>9</v>
       </c>
@@ -4708,7 +4712,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="64" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>9</v>
       </c>
@@ -4737,7 +4741,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="65" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>9</v>
       </c>
@@ -4766,7 +4770,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="66" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>9</v>
       </c>
@@ -4795,7 +4799,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="67" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>9</v>
       </c>
@@ -4824,7 +4828,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="68" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>9</v>
       </c>
@@ -4853,7 +4857,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="69" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>9</v>
       </c>
@@ -4882,7 +4886,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="70" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>9</v>
       </c>
@@ -4911,7 +4915,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="71" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>9</v>
       </c>
@@ -4940,7 +4944,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="72" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>9</v>
       </c>
@@ -4969,7 +4973,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="73" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>9</v>
       </c>
@@ -4998,7 +5002,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="74" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>9</v>
       </c>
@@ -5027,7 +5031,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="75" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>9</v>
       </c>
@@ -5056,7 +5060,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="76" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>9</v>
       </c>
@@ -5085,7 +5089,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="77" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>9</v>
       </c>
@@ -5114,7 +5118,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="78" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>9</v>
       </c>
@@ -5143,7 +5147,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="79" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>9</v>
       </c>
@@ -5172,7 +5176,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="80" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>9</v>
       </c>
@@ -5201,7 +5205,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="81" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>9</v>
       </c>
@@ -5230,7 +5234,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="82" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>9</v>
       </c>
@@ -5259,7 +5263,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="83" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>9</v>
       </c>
@@ -5288,7 +5292,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="84" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>9</v>
       </c>
@@ -5317,7 +5321,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="85" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>9</v>
       </c>
@@ -5346,7 +5350,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="86" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>9</v>
       </c>
@@ -5375,7 +5379,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="87" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>9</v>
       </c>
@@ -5404,7 +5408,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="88" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>9</v>
       </c>
@@ -5433,7 +5437,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="89" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>9</v>
       </c>
@@ -5462,7 +5466,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="90" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>9</v>
       </c>
@@ -5491,7 +5495,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="91" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>9</v>
       </c>
@@ -5520,7 +5524,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="92" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>9</v>
       </c>
@@ -5549,7 +5553,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="93" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>9</v>
       </c>
@@ -5578,7 +5582,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="94" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>9</v>
       </c>
@@ -5607,7 +5611,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="95" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>9</v>
       </c>
@@ -5636,7 +5640,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="96" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>9</v>
       </c>
@@ -5665,7 +5669,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="97" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>9</v>
       </c>
@@ -5694,7 +5698,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="98" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>9</v>
       </c>
@@ -5723,7 +5727,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="99" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>9</v>
       </c>
@@ -5752,7 +5756,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="100" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>9</v>
       </c>
@@ -5781,7 +5785,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="101" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>9</v>
       </c>
@@ -5810,7 +5814,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="102" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>9</v>
       </c>
@@ -5839,7 +5843,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="103" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>9</v>
       </c>
@@ -5868,7 +5872,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="104" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>9</v>
       </c>
@@ -5897,7 +5901,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="105" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>9</v>
       </c>
@@ -5926,7 +5930,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="106" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>9</v>
       </c>
@@ -5955,7 +5959,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="107" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>9</v>
       </c>
@@ -5984,7 +5988,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="108" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>9</v>
       </c>
@@ -6013,7 +6017,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="109" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>9</v>
       </c>
@@ -6042,7 +6046,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="110" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>9</v>
       </c>
@@ -6071,7 +6075,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="111" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>9</v>
       </c>
@@ -6100,7 +6104,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="112" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>9</v>
       </c>
@@ -6129,7 +6133,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="113" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>9</v>
       </c>
@@ -6158,7 +6162,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="114" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>9</v>
       </c>
@@ -6187,7 +6191,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="115" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>9</v>
       </c>
@@ -6216,7 +6220,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="116" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>9</v>
       </c>
@@ -6245,7 +6249,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="117" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>9</v>
       </c>
@@ -6274,7 +6278,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="118" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>9</v>
       </c>
@@ -6303,7 +6307,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="119" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>9</v>
       </c>
@@ -6332,7 +6336,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="120" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>9</v>
       </c>
@@ -6361,7 +6365,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="121" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>9</v>
       </c>
@@ -6390,7 +6394,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="122" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>9</v>
       </c>
@@ -6419,7 +6423,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="123" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>9</v>
       </c>
@@ -6448,7 +6452,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="124" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>9</v>
       </c>
@@ -6477,7 +6481,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="125" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>9</v>
       </c>
@@ -6506,7 +6510,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="126" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>9</v>
       </c>
@@ -6535,7 +6539,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="127" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>9</v>
       </c>
@@ -6564,7 +6568,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="128" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>9</v>
       </c>
@@ -6593,7 +6597,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="129" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>9</v>
       </c>
@@ -6622,7 +6626,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="130" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>9</v>
       </c>
@@ -6651,7 +6655,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="131" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>9</v>
       </c>
@@ -6680,7 +6684,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="132" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>9</v>
       </c>
@@ -6709,7 +6713,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="133" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>9</v>
       </c>
@@ -6738,7 +6742,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="134" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>9</v>
       </c>
@@ -6767,7 +6771,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="135" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>9</v>
       </c>
@@ -6796,7 +6800,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="136" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>9</v>
       </c>
@@ -6825,7 +6829,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="137" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>9</v>
       </c>
@@ -6854,7 +6858,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="138" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>9</v>
       </c>
@@ -6883,7 +6887,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="139" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>9</v>
       </c>
@@ -6912,7 +6916,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="140" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>9</v>
       </c>
@@ -6941,7 +6945,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="141" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>9</v>
       </c>
@@ -6970,7 +6974,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="142" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>9</v>
       </c>
@@ -6999,7 +7003,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="143" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>9</v>
       </c>
@@ -7028,7 +7032,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="144" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>9</v>
       </c>
@@ -7057,7 +7061,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="145" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>9</v>
       </c>
@@ -7086,7 +7090,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="146" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>9</v>
       </c>
@@ -7115,7 +7119,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="147" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>9</v>
       </c>
@@ -7144,7 +7148,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="148" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>9</v>
       </c>
@@ -7173,7 +7177,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="149" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>9</v>
       </c>
@@ -7202,7 +7206,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="150" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>9</v>
       </c>
@@ -7231,7 +7235,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="151" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>9</v>
       </c>
@@ -7260,7 +7264,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="152" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>9</v>
       </c>
@@ -7289,7 +7293,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="153" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>9</v>
       </c>
@@ -7318,7 +7322,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="154" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>9</v>
       </c>
@@ -7347,7 +7351,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="155" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>9</v>
       </c>
@@ -7376,7 +7380,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="156" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>9</v>
       </c>
@@ -7405,7 +7409,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="157" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>9</v>
       </c>
@@ -7434,7 +7438,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="158" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>9</v>
       </c>
@@ -7463,7 +7467,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="159" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>9</v>
       </c>
@@ -7492,7 +7496,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="160" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>9</v>
       </c>
@@ -7521,7 +7525,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="161" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>9</v>
       </c>
@@ -7550,7 +7554,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="162" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>9</v>
       </c>
@@ -7579,7 +7583,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="163" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>9</v>
       </c>
@@ -7608,7 +7612,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="164" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>9</v>
       </c>
@@ -7637,7 +7641,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="165" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>9</v>
       </c>
@@ -7666,7 +7670,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="166" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>9</v>
       </c>
@@ -7695,7 +7699,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="167" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>9</v>
       </c>
@@ -7724,7 +7728,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="168" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>9</v>
       </c>
@@ -7753,7 +7757,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="169" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>9</v>
       </c>
@@ -7782,7 +7786,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="170" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>9</v>
       </c>
@@ -7811,7 +7815,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="171" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>9</v>
       </c>
@@ -7840,7 +7844,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="172" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>9</v>
       </c>
@@ -7869,7 +7873,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="173" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>9</v>
       </c>
@@ -7898,7 +7902,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="174" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>9</v>
       </c>
@@ -7927,7 +7931,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="175" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>9</v>
       </c>
@@ -7956,7 +7960,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="176" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>9</v>
       </c>
@@ -7985,7 +7989,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="177" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>9</v>
       </c>
@@ -8014,7 +8018,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="178" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>9</v>
       </c>
@@ -8043,7 +8047,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="179" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>9</v>
       </c>
@@ -8072,7 +8076,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="180" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>9</v>
       </c>
@@ -8101,7 +8105,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="181" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>9</v>
       </c>
@@ -8130,7 +8134,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="182" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>9</v>
       </c>
@@ -8159,7 +8163,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="183" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>9</v>
       </c>
@@ -8188,7 +8192,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="184" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>9</v>
       </c>
@@ -8217,7 +8221,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="185" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>9</v>
       </c>
@@ -8246,7 +8250,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="186" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>9</v>
       </c>
@@ -8275,7 +8279,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="187" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>9</v>
       </c>
@@ -8304,7 +8308,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="188" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>9</v>
       </c>
@@ -8333,7 +8337,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="189" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>9</v>
       </c>
@@ -8362,7 +8366,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="190" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>9</v>
       </c>
@@ -8391,7 +8395,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="191" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>9</v>
       </c>
@@ -8420,7 +8424,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="192" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>9</v>
       </c>
@@ -8449,7 +8453,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="193" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>9</v>
       </c>
@@ -8478,7 +8482,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="194" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>9</v>
       </c>
@@ -8507,7 +8511,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="195" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>9</v>
       </c>
@@ -8536,7 +8540,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="196" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>9</v>
       </c>
@@ -8565,7 +8569,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="197" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>9</v>
       </c>
@@ -8594,7 +8598,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="198" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>9</v>
       </c>
@@ -8623,7 +8627,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="199" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>9</v>
       </c>
@@ -8652,7 +8656,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="200" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>9</v>
       </c>
@@ -8681,7 +8685,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="201" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>9</v>
       </c>
@@ -8710,7 +8714,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="202" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>9</v>
       </c>
@@ -8739,7 +8743,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="203" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>9</v>
       </c>
@@ -8768,7 +8772,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="204" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>9</v>
       </c>
@@ -8797,7 +8801,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="205" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>9</v>
       </c>
@@ -8826,7 +8830,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="206" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>9</v>
       </c>
@@ -8855,7 +8859,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="207" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>9</v>
       </c>
@@ -8884,7 +8888,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="208" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>9</v>
       </c>
@@ -8913,7 +8917,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="209" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>9</v>
       </c>
@@ -8942,7 +8946,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="210" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>9</v>
       </c>
@@ -8971,7 +8975,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="211" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>9</v>
       </c>
@@ -9000,7 +9004,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="212" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>9</v>
       </c>
@@ -9029,7 +9033,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="213" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>9</v>
       </c>
@@ -9058,7 +9062,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="214" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>9</v>
       </c>
@@ -9087,7 +9091,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="215" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>9</v>
       </c>
@@ -9116,7 +9120,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="216" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>9</v>
       </c>
@@ -9145,7 +9149,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="217" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>9</v>
       </c>
@@ -9174,7 +9178,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="218" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>9</v>
       </c>
@@ -9203,7 +9207,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="219" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>9</v>
       </c>
@@ -9232,7 +9236,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="220" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>9</v>
       </c>
@@ -9261,7 +9265,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="221" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>9</v>
       </c>
@@ -9290,7 +9294,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="222" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>9</v>
       </c>
@@ -9319,7 +9323,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="223" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>9</v>
       </c>
@@ -9348,7 +9352,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="224" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>9</v>
       </c>
@@ -9377,7 +9381,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="225" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>9</v>
       </c>
@@ -9406,7 +9410,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="226" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>9</v>
       </c>
@@ -9435,7 +9439,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="227" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>9</v>
       </c>
@@ -9464,7 +9468,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="228" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>9</v>
       </c>
@@ -9493,7 +9497,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="229" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>9</v>
       </c>
@@ -9522,7 +9526,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="230" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>9</v>
       </c>
@@ -9551,7 +9555,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="231" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>9</v>
       </c>
@@ -9580,7 +9584,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="232" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>9</v>
       </c>
@@ -9609,7 +9613,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="233" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>9</v>
       </c>
@@ -9638,7 +9642,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="234" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>9</v>
       </c>
@@ -9667,7 +9671,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="235" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>9</v>
       </c>
@@ -9696,7 +9700,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="236" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>9</v>
       </c>
@@ -9725,7 +9729,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="237" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>9</v>
       </c>
@@ -9754,7 +9758,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="238" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>9</v>
       </c>
@@ -9783,7 +9787,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="239" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>9</v>
       </c>
@@ -9812,7 +9816,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="240" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>9</v>
       </c>
@@ -9841,7 +9845,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="241" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>9</v>
       </c>
@@ -9870,7 +9874,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="242" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>9</v>
       </c>
@@ -9899,7 +9903,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="243" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>9</v>
       </c>
@@ -9928,7 +9932,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="244" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>9</v>
       </c>
@@ -9957,7 +9961,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="245" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>9</v>
       </c>
@@ -9986,7 +9990,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="246" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>9</v>
       </c>
@@ -10015,7 +10019,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="247" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>9</v>
       </c>
@@ -10044,7 +10048,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="248" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>9</v>
       </c>
@@ -10073,7 +10077,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="249" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>9</v>
       </c>
@@ -10102,7 +10106,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="250" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>9</v>
       </c>
@@ -10131,7 +10135,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="251" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>9</v>
       </c>
@@ -10160,7 +10164,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="252" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>9</v>
       </c>
@@ -10189,7 +10193,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="253" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>9</v>
       </c>
@@ -10218,7 +10222,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="254" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>9</v>
       </c>
@@ -10247,7 +10251,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="255" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>9</v>
       </c>
@@ -10276,7 +10280,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="256" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>9</v>
       </c>
@@ -10305,7 +10309,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="257" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>9</v>
       </c>
@@ -10334,7 +10338,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="258" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
         <v>9</v>
       </c>
@@ -10363,7 +10367,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="259" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>9</v>
       </c>
@@ -10392,7 +10396,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="260" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>9</v>
       </c>
@@ -10421,7 +10425,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="261" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>9</v>
       </c>
@@ -10450,7 +10454,7 @@
         <v>702</v>
       </c>
     </row>
-    <row r="262" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>9</v>
       </c>
@@ -10479,7 +10483,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="263" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>9</v>
       </c>
@@ -10508,7 +10512,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="264" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>9</v>
       </c>
@@ -10537,7 +10541,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="265" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>9</v>
       </c>
@@ -10566,7 +10570,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="266" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
         <v>9</v>
       </c>
@@ -10595,7 +10599,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="267" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>9</v>
       </c>
@@ -10624,7 +10628,7 @@
         <v>716</v>
       </c>
     </row>
-    <row r="268" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
         <v>9</v>
       </c>
@@ -10653,7 +10657,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="269" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
         <v>9</v>
       </c>
@@ -10682,7 +10686,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="270" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A270" t="s">
         <v>9</v>
       </c>
@@ -10711,7 +10715,7 @@
         <v>722</v>
       </c>
     </row>
-    <row r="271" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
         <v>9</v>
       </c>
@@ -10740,7 +10744,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="272" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A272" t="s">
         <v>9</v>
       </c>
@@ -10769,7 +10773,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="273" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
         <v>9</v>
       </c>
@@ -10798,7 +10802,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="274" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
         <v>9</v>
       </c>
@@ -10827,7 +10831,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="275" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
         <v>9</v>
       </c>
@@ -10856,7 +10860,7 @@
         <v>732</v>
       </c>
     </row>
-    <row r="276" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A276" t="s">
         <v>9</v>
       </c>
@@ -10885,7 +10889,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="277" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A277" t="s">
         <v>9</v>
       </c>
@@ -10914,7 +10918,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="278" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
         <v>9</v>
       </c>
@@ -10943,7 +10947,7 @@
         <v>738</v>
       </c>
     </row>
-    <row r="279" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>9</v>
       </c>
@@ -10972,7 +10976,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="280" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
         <v>9</v>
       </c>
@@ -11001,7 +11005,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="281" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
         <v>9</v>
       </c>
@@ -11030,7 +11034,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="282" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
         <v>9</v>
       </c>
@@ -11059,7 +11063,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="283" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
         <v>9</v>
       </c>
@@ -11088,7 +11092,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="284" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
         <v>9</v>
       </c>
@@ -11117,7 +11121,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="285" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
         <v>9</v>
       </c>
@@ -11146,7 +11150,7 @@
         <v>755</v>
       </c>
     </row>
-    <row r="286" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
         <v>9</v>
       </c>
@@ -11175,7 +11179,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="287" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
         <v>9</v>
       </c>
@@ -11204,7 +11208,7 @@
         <v>759</v>
       </c>
     </row>
-    <row r="288" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
         <v>9</v>
       </c>
@@ -11233,7 +11237,7 @@
         <v>761</v>
       </c>
     </row>
-    <row r="289" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
         <v>9</v>
       </c>
@@ -11262,7 +11266,7 @@
         <v>763</v>
       </c>
     </row>
-    <row r="290" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A290" t="s">
         <v>9</v>
       </c>
@@ -11291,7 +11295,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="291" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
         <v>9</v>
       </c>
@@ -11320,7 +11324,7 @@
         <v>767</v>
       </c>
     </row>
-    <row r="292" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A292" t="s">
         <v>9</v>
       </c>
@@ -11349,7 +11353,7 @@
         <v>769</v>
       </c>
     </row>
-    <row r="293" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A293" t="s">
         <v>9</v>
       </c>
@@ -11378,7 +11382,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="294" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A294" t="s">
         <v>9</v>
       </c>
@@ -11407,7 +11411,7 @@
         <v>773</v>
       </c>
     </row>
-    <row r="295" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A295" t="s">
         <v>9</v>
       </c>
@@ -11436,7 +11440,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="296" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
         <v>9</v>
       </c>
@@ -11465,7 +11469,7 @@
         <v>778</v>
       </c>
     </row>
-    <row r="297" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A297" t="s">
         <v>9</v>
       </c>
@@ -11494,7 +11498,7 @@
         <v>780</v>
       </c>
     </row>
-    <row r="298" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
         <v>9</v>
       </c>
@@ -11523,7 +11527,7 @@
         <v>782</v>
       </c>
     </row>
-    <row r="299" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
         <v>9</v>
       </c>
@@ -11552,7 +11556,7 @@
         <v>784</v>
       </c>
     </row>
-    <row r="300" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A300" t="s">
         <v>9</v>
       </c>
@@ -11581,7 +11585,7 @@
         <v>786</v>
       </c>
     </row>
-    <row r="301" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
         <v>9</v>
       </c>
@@ -11610,7 +11614,7 @@
         <v>788</v>
       </c>
     </row>
-    <row r="302" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>9</v>
       </c>
@@ -11639,7 +11643,7 @@
         <v>790</v>
       </c>
     </row>
-    <row r="303" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>9</v>
       </c>
@@ -11668,7 +11672,7 @@
         <v>792</v>
       </c>
     </row>
-    <row r="304" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>9</v>
       </c>
@@ -11697,7 +11701,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="305" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
         <v>9</v>
       </c>
@@ -11726,7 +11730,7 @@
         <v>796</v>
       </c>
     </row>
-    <row r="306" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>9</v>
       </c>
@@ -11755,9 +11759,9 @@
         <v>798</v>
       </c>
     </row>
-    <row r="307" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
-        <v>799</v>
+        <v>9</v>
       </c>
       <c r="B307" t="s">
         <v>800</v>
@@ -11784,9 +11788,9 @@
         <v>802</v>
       </c>
     </row>
-    <row r="308" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
-        <v>799</v>
+        <v>9</v>
       </c>
       <c r="B308" t="s">
         <v>803</v>
@@ -11813,9 +11817,9 @@
         <v>804</v>
       </c>
     </row>
-    <row r="309" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A309" t="s">
-        <v>799</v>
+        <v>9</v>
       </c>
       <c r="B309" t="s">
         <v>805</v>
@@ -11842,9 +11846,9 @@
         <v>806</v>
       </c>
     </row>
-    <row r="310" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A310" t="s">
-        <v>799</v>
+        <v>9</v>
       </c>
       <c r="B310" t="s">
         <v>807</v>
@@ -11871,9 +11875,9 @@
         <v>808</v>
       </c>
     </row>
-    <row r="311" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A311" t="s">
-        <v>799</v>
+        <v>9</v>
       </c>
       <c r="B311" t="s">
         <v>809</v>
@@ -11900,7 +11904,7 @@
         <v>810</v>
       </c>
     </row>
-    <row r="312" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A312" t="s">
         <v>799</v>
       </c>
@@ -11929,7 +11933,7 @@
         <v>812</v>
       </c>
     </row>
-    <row r="313" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A313" t="s">
         <v>799</v>
       </c>
@@ -11958,9 +11962,9 @@
         <v>814</v>
       </c>
     </row>
-    <row r="314" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A314" t="s">
-        <v>799</v>
+        <v>9</v>
       </c>
       <c r="B314" t="s">
         <v>815</v>
@@ -11987,9 +11991,9 @@
         <v>816</v>
       </c>
     </row>
-    <row r="315" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A315" t="s">
-        <v>799</v>
+        <v>9</v>
       </c>
       <c r="B315" t="s">
         <v>817</v>
@@ -12017,10 +12021,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I315" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:I315" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="NV"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:I315" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:I306 A312:I313 B307:I307 B308:I311 B315:I315 B314:I314" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -12028,14 +12038,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.796875" customWidth="1"/>
     <col min="2" max="2" width="48.796875" customWidth="1"/>
     <col min="3" max="3" width="110.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>819</v>
       </c>
@@ -12046,7 +12056,7 @@
         <v>821</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>822</v>
       </c>

</xml_diff>

<commit_message>
updated code for plan search scripts
</commit_message>
<xml_diff>
--- a/data/marketplace/MarketplacePlansData.xlsx
+++ b/data/marketplace/MarketplacePlansData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://molinahealthcare-my.sharepoint.com/personal/naresh_jangid_molinahealthcare_com/Documents/Automation/molina_automation/marketplace/data/marketplace/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="11_70CE30217927462588B21A62D89D467537775006" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B15F36B0-41C2-4005-9C8F-EE767325F417}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="11_0CF6D607091F0106E0C21E1DAC55B2F500AFEF90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0FE2160D-FC22-4D66-A833-FA0CD05814D7}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -74,7 +74,7 @@
     <t>Schedule of Benefits</t>
   </si>
   <si>
-    <t>Molina Gold Core 1500</t>
+    <t>Schedule of Benefits – Molina Gold Core 1500</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_G1_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_G1_1.pdf</t>
@@ -83,7 +83,7 @@
     <t>TC002 Molina Gold Core Zero OH-2027</t>
   </si>
   <si>
-    <t>Molina Gold Core Zero</t>
+    <t>Schedule of Benefits – Molina Gold Core Zero</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_G1_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_G1_2.pdf</t>
@@ -92,7 +92,7 @@
     <t>TC003 Molina Gold Core 1500 LCS OH-2027</t>
   </si>
   <si>
-    <t>Molina Gold Core 1500 LCS</t>
+    <t>Schedule of Benefits – Molina Gold Core 1500 LCS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_G1_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_G1_3.pdf</t>
@@ -101,7 +101,7 @@
     <t>TC004 Molina Silver Core 70 OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Core 70</t>
+    <t>Schedule of Benefits – Molina Silver Core 70</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S1_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S1_1.pdf</t>
@@ -110,7 +110,7 @@
     <t>TC005 Molina Silver Core Zero OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Core Zero</t>
+    <t>Schedule of Benefits – Molina Silver Core Zero</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S1_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S1_2.pdf</t>
@@ -119,7 +119,7 @@
     <t>TC006 Molina Silver Core LCS OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Core LCS</t>
+    <t>Schedule of Benefits – Molina Silver Core LCS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S1_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S1_3.pdf</t>
@@ -128,7 +128,7 @@
     <t>TC007 Molina Silver Core 73 OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Core 73</t>
+    <t>Schedule of Benefits – Molina Silver Core 73</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S1_4.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S1_4.pdf</t>
@@ -137,7 +137,7 @@
     <t>TC008 Molina Silver Core 87 OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Core 87</t>
+    <t>Schedule of Benefits – Molina Silver Core 87</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S1_5.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S1_5.pdf</t>
@@ -146,7 +146,7 @@
     <t>TC009 Molina Silver Core 94 OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Core 94</t>
+    <t>Schedule of Benefits – Molina Silver Core 94</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S1_6.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S1_6.pdf</t>
@@ -155,7 +155,7 @@
     <t>TC010 Molina Silver Saver 70 with Four Free PCP Visits OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Saver 70 with Four Free PCP Visits</t>
+    <t>Schedule of Benefits – Molina Silver Saver 70 with Four Free PCP Visits</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S12_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S12_1.pdf</t>
@@ -164,7 +164,7 @@
     <t>TC011 Molina Silver Saver Zero OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Saver Zero</t>
+    <t>Schedule of Benefits – Molina Silver Saver Zero</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S12_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S12_2.pdf</t>
@@ -173,7 +173,7 @@
     <t>TC012 Molina Silver Saver LCS with Four Free PCP Visits OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Saver LCS with Four Free PCP Visits</t>
+    <t>Schedule of Benefits – Molina Silver Saver LCS with Four Free PCP Visits</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S12_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S12_3.pdf</t>
@@ -182,7 +182,7 @@
     <t>TC013 Molina Silver Saver 73 with Four Free PCP Visits OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Saver 73 with Four Free PCP Visits</t>
+    <t>Schedule of Benefits – Molina Silver Saver 73 with Four Free PCP Visits</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S12_4.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S12_4.pdf</t>
@@ -191,7 +191,7 @@
     <t>TC014 Molina Silver Saver 87 with Four Free PCP Visits OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Saver 87 with Four Free PCP Visits</t>
+    <t>Schedule of Benefits – Molina Silver Saver 87 with Four Free PCP Visits</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S12_5.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S12_5.pdf</t>
@@ -200,7 +200,7 @@
     <t>TC015 Molina Silver Saver 94 with Four Free PCP Visits OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Saver 94 with Four Free PCP Visits</t>
+    <t>Schedule of Benefits – Molina Silver Saver 94 with Four Free PCP Visits</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S12_6.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S12_6.pdf</t>
@@ -209,7 +209,7 @@
     <t>TC016 Molina Bronze Saver 7000 OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Saver 7000</t>
+    <t>Schedule of Benefits – Molina Bronze Saver 7000</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_B12V_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_B12V_1.pdf</t>
@@ -218,7 +218,7 @@
     <t>TC017 Molina Bronze Saver Zero OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Saver Zero</t>
+    <t>Schedule of Benefits – Molina Bronze Saver Zero</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_B12V_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_B12V_2.pdf</t>
@@ -227,7 +227,7 @@
     <t>TC018 Molina Bronze Saver 7000 LCS OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Saver 7000 LCS</t>
+    <t>Schedule of Benefits – Molina Bronze Saver 7000 LCS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_B12V_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_B12V_3.pdf</t>
@@ -236,7 +236,7 @@
     <t>TC019 Molina Bronze Enhanced 4000 OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Enhanced 4000</t>
+    <t>Schedule of Benefits – Molina Bronze Enhanced 4000</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_B10V_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_B10V_1.pdf</t>
@@ -245,7 +245,7 @@
     <t>TC020 Molina Bronze Enhanced Zero OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Enhanced Zero</t>
+    <t>Schedule of Benefits – Molina Bronze Enhanced Zero</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_B10V_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_B10V_2.pdf</t>
@@ -254,7 +254,7 @@
     <t>TC021 Molina Bronze Enhanced 4000 LCS OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Enhanced 4000 LCS</t>
+    <t>Schedule of Benefits – Molina Bronze Enhanced 4000 LCS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_B10V_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_B10V_3.pdf</t>
@@ -263,7 +263,7 @@
     <t>TC022 Molina Gold Enhanced 895 OH-2027</t>
   </si>
   <si>
-    <t>Molina Gold Enhanced 895</t>
+    <t>Schedule of Benefits – Molina Gold Enhanced 895</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_G9V_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_G9V_1.pdf</t>
@@ -272,7 +272,7 @@
     <t>TC023 Molina Gold Enhanced Zero OH-2027</t>
   </si>
   <si>
-    <t>Molina Gold Enhanced Zero</t>
+    <t>Schedule of Benefits – Molina Gold Enhanced Zero</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_G9V_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_G9V_2.pdf</t>
@@ -281,7 +281,7 @@
     <t>TC024 Molina Gold Enhanced 895 LCS OH-2027</t>
   </si>
   <si>
-    <t>Molina Gold Enhanced 895 LCS</t>
+    <t>Schedule of Benefits – Molina Gold Enhanced 895 LCS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_G9V_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_G9V_3.pdf</t>
@@ -290,7 +290,7 @@
     <t>TC025 Molina Silver Empower 2750 OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Empower 2750</t>
+    <t>Schedule of Benefits – Molina Silver Empower 2750</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S16V_0.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S16V_0.pdf</t>
@@ -299,7 +299,7 @@
     <t>TC026 Molina Silver Empower 3750 OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Empower 3750</t>
+    <t>Schedule of Benefits – Molina Silver Empower 3750</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S17V_0.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S17V_0.pdf</t>
@@ -308,7 +308,7 @@
     <t>TC027 Molina Silver Empower 4500 OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Empower 4500</t>
+    <t>Schedule of Benefits – Molina Silver Empower 4500</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S18V_0.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S18V_0.pdf</t>
@@ -317,7 +317,7 @@
     <t>TC028 Molina Silver Empower 5500 OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Empower 5500</t>
+    <t>Schedule of Benefits – Molina Silver Empower 5500</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S19V_0.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S19V_0.pdf</t>
@@ -326,7 +326,7 @@
     <t>TC029 Molina Gold Empower 2000 OH-2027</t>
   </si>
   <si>
-    <t>Molina Gold Empower 2000</t>
+    <t>Schedule of Benefits – Molina Gold Empower 2000</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_G16V_0.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_G16V_0.pdf</t>
@@ -335,7 +335,7 @@
     <t>TC030 Molina Bronze Empower 6000 OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Empower 6000</t>
+    <t>Schedule of Benefits – Molina Bronze Empower 6000</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_B16V_0.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_B16V_0.pdf</t>
@@ -344,7 +344,7 @@
     <t>TC031 Molina Gold Core 1500 Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Gold Core 1500 Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Gold Core 1500 Plus with Adult Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_G1V_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_G1V_1.pdf</t>
@@ -353,7 +353,7 @@
     <t>TC032 Molina Gold Core Zero Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Gold Core Zero Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Gold Core Zero Plus with Adult Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_G1V_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_G1V_2.pdf</t>
@@ -362,7 +362,7 @@
     <t>TC033 Molina Gold Core 1500 LCS Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Gold Core 1500 LCS Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Gold Core 1500 LCS Plus with Adult Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_G1V_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_G1V_3.pdf</t>
@@ -371,7 +371,7 @@
     <t>TC034 Molina Silver Core 70 Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Core 70 Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Silver Core 70 Plus with Adult Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S1V_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S1V_1.pdf</t>
@@ -380,7 +380,7 @@
     <t>TC035 Molina Silver Core Zero Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Core Zero Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Silver Core Zero Plus with Adult Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S1V_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S1V_2.pdf</t>
@@ -389,7 +389,7 @@
     <t>TC036 Molina Silver Core LCS Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Core LCS Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Silver Core LCS Plus with Adult Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S1V_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S1V_3.pdf</t>
@@ -398,7 +398,7 @@
     <t>TC037 Molina Silver Core 73 Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Core 73 Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Silver Core 73 Plus with Adult Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S1V_4.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S1V_4.pdf</t>
@@ -407,7 +407,7 @@
     <t>TC038 Molina Silver Core 87 Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Core 87 Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Silver Core 87 Plus with Adult Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S1V_5.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S1V_5.pdf</t>
@@ -416,7 +416,7 @@
     <t>TC039 Molina Silver Core 94 Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Core 94 Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Silver Core 94 Plus with Adult Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S1V_6.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S1V_6.pdf</t>
@@ -425,97 +425,97 @@
     <t>TC040 Molina Bronze Enhanced 4000 Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Enhanced 4000 Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Bronze Enhanced 4000 Plus with Adult Vision</t>
   </si>
   <si>
     <t>TC041 Molina Bronze Enhanced Zero Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Enhanced Zero Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Bronze Enhanced Zero Plus with Adult Vision</t>
   </si>
   <si>
     <t>TC042 Molina Bronze Enhanced 4000 LCS Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Enhanced 4000 LCS Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Bronze Enhanced 4000 LCS Plus with Adult Vision</t>
   </si>
   <si>
     <t>TC043 Molina Gold Enhanced 895 Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Gold Enhanced 895 Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Gold Enhanced 895 Plus with Adult Vision</t>
   </si>
   <si>
     <t>TC044 Molina Gold Enhanced Zero Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Gold Enhanced Zero Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Gold Enhanced Zero Plus with Adult Vision</t>
   </si>
   <si>
     <t>TC045 Molina Gold Enhanced 895 LCS Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Gold Enhanced 895 LCS Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Gold Enhanced 895 LCS Plus with Adult Vision</t>
   </si>
   <si>
     <t>TC046 Molina Silver Empower 2750 Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Empower 2750 Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Silver Empower 2750 Plus with Adult Vision</t>
   </si>
   <si>
     <t>TC047 Molina Silver Empower 3750 Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Empower 3750 Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Silver Empower 3750 Plus with Adult Vision</t>
   </si>
   <si>
     <t>TC048 Molina Silver Empower 4500 Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Empower 4500 Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Silver Empower 4500 Plus with Adult Vision</t>
   </si>
   <si>
     <t>TC049 Molina Silver Empower 5500 Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Empower 5500 Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Silver Empower 5500 Plus with Adult Vision</t>
   </si>
   <si>
     <t>TC050 Molina Gold Empower 2000 Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Gold Empower 2000 Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Gold Empower 2000 Plus with Adult Vision</t>
   </si>
   <si>
     <t>TC051 Molina Bronze Empower 6000 Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Empower 6000 Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Bronze Empower 6000 Plus with Adult Vision</t>
   </si>
   <si>
     <t>TC052 Molina Bronze Saver 7000 Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Saver 7000 Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Bronze Saver 7000 Plus with Adult Vision</t>
   </si>
   <si>
     <t>TC053 Molina Bronze Saver Zero Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Saver Zero Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Bronze Saver Zero Plus with Adult Vision</t>
   </si>
   <si>
     <t>TC054 Molina Bronze Saver 7000 LCS Plus with Adult Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Saver 7000 LCS Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Bronze Saver 7000 LCS Plus with Adult Vision</t>
   </si>
   <si>
     <t>TC055 Molina Gold Core 1500 Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Gold Core 1500 Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Gold Core 1500 Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_G1DV_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_G1DV_1.pdf</t>
@@ -524,7 +524,7 @@
     <t>TC056 Molina Gold Core Zero Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Gold Core Zero Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Gold Core Zero Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_G1DV_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_G1DV_2.pdf</t>
@@ -533,7 +533,7 @@
     <t>TC057 Molina Gold Core 1500 LCS Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Gold Core 1500 LCS Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Gold Core 1500 LCS Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_G1DV_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_G1DV_3.pdf</t>
@@ -542,7 +542,7 @@
     <t>TC058 Molina Silver Core 70 Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Core 70 Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Silver Core 70 Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S1DV_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S1DV_1.pdf</t>
@@ -551,7 +551,7 @@
     <t>TC059 Molina Silver Core Zero Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Core Zero Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Silver Core Zero Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S1DV_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S1DV_2.pdf</t>
@@ -560,7 +560,7 @@
     <t>TC060 Molina Silver Core LCS Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Core LCS Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Silver Core LCS Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S1DV_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S1DV_3.pdf</t>
@@ -569,7 +569,7 @@
     <t>TC061 Molina Silver Core 73 Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Core 73 Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Silver Core 73 Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S1DV_4.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S1DV_4.pdf</t>
@@ -578,7 +578,7 @@
     <t>TC062 Molina Silver Core 87 Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Core 87 Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Silver Core 87 Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S1DV_5.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S1DV_5.pdf</t>
@@ -587,7 +587,7 @@
     <t>TC063 Molina Silver Core 94 Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Core 94 Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Silver Core 94 Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S1DV_6.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S1DV_6.pdf</t>
@@ -596,7 +596,7 @@
     <t>TC064 Molina Bronze Saver 7000 Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Saver 7000 Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Bronze Saver 7000 Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_B12DV_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_B12DV_1.pdf</t>
@@ -605,7 +605,7 @@
     <t>TC065 Molina Bronze Saver Zero Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Saver Zero Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Bronze Saver Zero Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_B12DV_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_B12DV_2.pdf</t>
@@ -614,7 +614,7 @@
     <t>TC066 Molina Bronze Saver 7000 LCS Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Saver 7000 LCS Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Bronze Saver 7000 LCS Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_B12DV_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_B12DV_3.pdf</t>
@@ -623,7 +623,7 @@
     <t>TC067 Molina Bronze Enhanced 4000 Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Enhanced 4000 Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Bronze Enhanced 4000 Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_B10DV_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_B10DV_1.pdf</t>
@@ -632,7 +632,7 @@
     <t>TC068 Molina Bronze Enhanced Zero Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Enhanced Zero Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Bronze Enhanced Zero Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_B10DV_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_B10DV_2.pdf</t>
@@ -641,7 +641,7 @@
     <t>TC069 Molina Bronze Enhanced 4000 LCS Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Enhanced 4000 LCS Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Bronze Enhanced 4000 LCS Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_B10DV_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_B10DV_3.pdf</t>
@@ -650,7 +650,7 @@
     <t>TC070 Molina Gold Enhanced 895 Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Gold Enhanced 895 Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Gold Enhanced 895 Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_G9DV_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_G9DV_1.pdf</t>
@@ -659,7 +659,7 @@
     <t>TC071 Molina Gold Enhanced Zero Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Gold Enhanced Zero Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Gold Enhanced Zero Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_G9DV_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_G9DV_2.pdf</t>
@@ -668,7 +668,7 @@
     <t>TC072 Molina Gold Enhanced 895 LCS Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Gold Enhanced 895 LCS Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Gold Enhanced 895 LCS Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_G9DV_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_G9DV_3.pdf</t>
@@ -677,7 +677,7 @@
     <t>TC073 Molina Silver Empower 2750 Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Empower 2750 Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Silver Empower 2750 Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S16DV_0.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S16DV_0.pdf</t>
@@ -686,7 +686,7 @@
     <t>TC074 Molina Silver Empower 3750 Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Empower 3750 Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Silver Empower 3750 Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S17DV_0.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S17DV_0.pdf</t>
@@ -695,7 +695,7 @@
     <t>TC075 Molina Silver Empower 4500 Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Empower 4500 Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Silver Empower 4500 Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S18DV_0.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S18DV_0.pdf</t>
@@ -704,7 +704,7 @@
     <t>TC076 Molina Silver Empower 5500 Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Empower 5500 Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Silver Empower 5500 Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S19DV_0.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S19DV_0.pdf</t>
@@ -713,7 +713,7 @@
     <t>TC077 Molina Gold Empower 2000 Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Gold Empower 2000 Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Gold Empower 2000 Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_G16DV_0.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_G16DV_0.pdf</t>
@@ -722,7 +722,7 @@
     <t>TC078 Molina Bronze Empower 6000 Plus with Adult Dental and Vision OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Empower 6000 Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Bronze Empower 6000 Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_B16DV_0.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_B16DV_0.pdf</t>
@@ -731,7 +731,7 @@
     <t>TC079 Molina Bronze Smart Heart Health OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Smart Heart Health</t>
+    <t>Schedule of Benefits – Molina Bronze Smart Heart Health</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_B15_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_B15_1.pdf</t>
@@ -740,7 +740,7 @@
     <t>TC080 Molina Bronze Smart Zero Heart Health OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Smart Zero Heart Health</t>
+    <t>Schedule of Benefits – Molina Bronze Smart Zero Heart Health</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_B15_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_B15_2.pdf</t>
@@ -749,7 +749,7 @@
     <t>TC081 Molina Bronze Smart LCS Heart Health OH-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Smart LCS Heart Health</t>
+    <t>Schedule of Benefits – Molina Bronze Smart LCS Heart Health</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_B15_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_B15_3.pdf</t>
@@ -758,7 +758,7 @@
     <t>TC082 Molina Silver Smart 70 Heart Health OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Smart 70 Heart Health</t>
+    <t>Schedule of Benefits – Molina Silver Smart 70 Heart Health</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S15_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S15_1.pdf</t>
@@ -767,7 +767,7 @@
     <t>TC083 Molina Silver Smart Zero Heart Health OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Smart Zero Heart Health</t>
+    <t>Schedule of Benefits – Molina Silver Smart Zero Heart Health</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S15_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S15_2.pdf</t>
@@ -776,7 +776,7 @@
     <t>TC084 Molina Silver Smart LCS Heart Health OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Smart LCS Heart Health</t>
+    <t>Schedule of Benefits – Molina Silver Smart LCS Heart Health</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S15_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S15_3.pdf</t>
@@ -785,7 +785,7 @@
     <t>TC085 Molina Silver Smart 73 Heart Health OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Smart 73 Heart Health</t>
+    <t>Schedule of Benefits – Molina Silver Smart 73 Heart Health</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S15_4.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S15_4.pdf</t>
@@ -794,7 +794,7 @@
     <t>TC086 Molina Silver Smart 87 Heart Health OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Smart 87 Heart Health</t>
+    <t>Schedule of Benefits – Molina Silver Smart 87 Heart Health</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S15_5.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S15_5.pdf</t>
@@ -803,7 +803,7 @@
     <t>TC087 Molina Silver Smart 94 Heart Health OH-2027</t>
   </si>
   <si>
-    <t>Molina Silver Smart 94 Heart Health</t>
+    <t>Schedule of Benefits – Molina Silver Smart 94 Heart Health</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/english/OH26SOBE_S15_6.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/oh/materials/SOB/2027/spanish/OH26SOBS_S15_6.pdf</t>
@@ -1016,7 +1016,7 @@
     <t>CA</t>
   </si>
   <si>
-    <t>Bronze 60 HMO</t>
+    <t>Schedule of Benefits – Bronze 60 HMO</t>
   </si>
   <si>
     <t>https://pws-q3.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/ca/materials/SOB/2027/english/CA27SOBE_B60_1.pdf|https://pws-q3.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/ca/materials/SOB/2027/spanish/CA27SOBS_B60_1.pdf</t>
@@ -1025,7 +1025,7 @@
     <t>TC122 $0 Cost Share HMO AI-AN CA-2027</t>
   </si>
   <si>
-    <t>$0 Cost Share HMO AI-AN</t>
+    <t>Schedule of Benefits – $0 Cost Share HMO AI-AN</t>
   </si>
   <si>
     <t/>
@@ -1034,67 +1034,67 @@
     <t>TC123 Bronze 60 HMO AI-AN CA-2027</t>
   </si>
   <si>
-    <t>Bronze 60 HMO AI-AN</t>
+    <t>Schedule of Benefits – Bronze 60 HMO AI-AN</t>
   </si>
   <si>
     <t>TC124 Gold 80 HMO CA-2027</t>
   </si>
   <si>
-    <t>Gold 80 HMO</t>
+    <t>Schedule of Benefits – Gold 80 HMO</t>
   </si>
   <si>
     <t>TC125 Gold 80 HMO AI-AN CA-2027</t>
   </si>
   <si>
-    <t>Gold 80 HMO AI-AN</t>
+    <t>Schedule of Benefits – Gold 80 HMO AI-AN</t>
   </si>
   <si>
     <t>TC126 Minimum Coverage HMO CA-2027</t>
   </si>
   <si>
-    <t>Minimum Coverage HMO</t>
+    <t>Schedule of Benefits – Minimum Coverage HMO</t>
   </si>
   <si>
     <t>TC127 Platinum 90 HMO CA-2027</t>
   </si>
   <si>
-    <t>Platinum 90 HMO</t>
+    <t>Schedule of Benefits – Platinum 90 HMO</t>
   </si>
   <si>
     <t>TC128 Platinum 90 HMO AI-AN CA-2027</t>
   </si>
   <si>
-    <t>Platinum 90 HMO AI-AN</t>
+    <t>Schedule of Benefits – Platinum 90 HMO AI-AN</t>
   </si>
   <si>
     <t>TC129 Silver 70 HMO CA-2027</t>
   </si>
   <si>
-    <t>Silver 70 HMO</t>
+    <t>Schedule of Benefits – Silver 70 HMO</t>
   </si>
   <si>
     <t>TC130 Silver 70 HMO AI-AN CA-2027</t>
   </si>
   <si>
-    <t>Silver 70 HMO AI-AN</t>
+    <t>Schedule of Benefits – Silver 70 HMO AI-AN</t>
   </si>
   <si>
     <t>TC131 Silver 73 HMO CA-2027</t>
   </si>
   <si>
-    <t>Silver 73 HMO</t>
+    <t>Schedule of Benefits – Silver 73 HMO</t>
   </si>
   <si>
     <t>TC132 Silver 87 HMO CA-2027</t>
   </si>
   <si>
-    <t>Silver 87 HMO</t>
+    <t>Schedule of Benefits – Silver 87 HMO</t>
   </si>
   <si>
     <t>TC133 Silver 94 HMO CA-2027</t>
   </si>
   <si>
-    <t>Silver 94 HMO</t>
+    <t>Schedule of Benefits – Silver 94 HMO</t>
   </si>
   <si>
     <t>TC134 Molina Cascade Complete Gold WA-2027</t>
@@ -1103,7 +1103,7 @@
     <t>WA</t>
   </si>
   <si>
-    <t>Molina Cascade Complete Gold</t>
+    <t>Schedule of Benefits – Molina Cascade Complete Gold</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/english/WA27SOBE_G6_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/spanish/WA27SOBS_G6_1.pdf</t>
@@ -1112,7 +1112,7 @@
     <t>TC135 Molina Cascade Complete Gold Zero WA-2027</t>
   </si>
   <si>
-    <t>Molina Cascade Complete Gold Zero</t>
+    <t>Schedule of Benefits – Molina Cascade Complete Gold Zero</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/english/WA27SOBE_G6_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/spanish/WA27SOBS_G6_2.pdf</t>
@@ -1121,7 +1121,7 @@
     <t>TC136 Molina Cascade Complete Gold LCS WA-2027</t>
   </si>
   <si>
-    <t>Molina Cascade Complete Gold LCS</t>
+    <t>Schedule of Benefits – Molina Cascade Complete Gold LCS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/english/WA27SOBE_G6_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/spanish/WA27SOBS_G6_3.pdf</t>
@@ -1130,7 +1130,7 @@
     <t>TC137 Molina Cascade Silver 70 WA-2027</t>
   </si>
   <si>
-    <t>Molina Cascade Silver 70</t>
+    <t>Schedule of Benefits – Molina Cascade Silver 70</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/english/WA27SOBE_S6_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/spanish/WA27SOBS_S6_1.pdf</t>
@@ -1139,7 +1139,7 @@
     <t>TC138 Molina Cascade Silver Zero WA-2027</t>
   </si>
   <si>
-    <t>Molina Cascade Silver Zero</t>
+    <t>Schedule of Benefits – Molina Cascade Silver Zero</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/english/WA27SOBE_S6_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/spanish/WA27SOBS_S6_2.pdf</t>
@@ -1148,7 +1148,7 @@
     <t>TC139 Molina Cascade Silver LCS WA-2027</t>
   </si>
   <si>
-    <t>Molina Cascade Silver LCS</t>
+    <t>Schedule of Benefits – Molina Cascade Silver LCS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/english/WA27SOBE_S6_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/spanish/WA27SOBS_S6_3.pdf</t>
@@ -1157,7 +1157,7 @@
     <t>TC140 Molina Cascade Silver 73 WA-2027</t>
   </si>
   <si>
-    <t>Molina Cascade Silver 73</t>
+    <t>Schedule of Benefits – Molina Cascade Silver 73</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/english/WA27SOBE_S6_4.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/spanish/WA27SOBS_S6_4.pdf</t>
@@ -1166,7 +1166,7 @@
     <t>TC141 Molina Cascade Silver 87 WA-2027</t>
   </si>
   <si>
-    <t>Molina Cascade Silver 87</t>
+    <t>Schedule of Benefits – Molina Cascade Silver 87</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/english/WA27SOBE_S6_5.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/spanish/WA27SOBS_S6_5.pdf</t>
@@ -1175,7 +1175,7 @@
     <t>TC142 Molina Cascade Silver 94 WA-2027</t>
   </si>
   <si>
-    <t>Molina Cascade Silver 94</t>
+    <t>Schedule of Benefits – Molina Cascade Silver 94</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/english/WA27SOBE_S6_6.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/spanish/WA27SOBS_S6_6.pdf</t>
@@ -1184,7 +1184,7 @@
     <t>TC143 Molina Cascade Bronze WA-2027</t>
   </si>
   <si>
-    <t>Molina Cascade Bronze</t>
+    <t>Schedule of Benefits – Molina Cascade Bronze</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/english/WA27SOBE_B6_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/spanish/WA27SOBS_B6_1.pdf</t>
@@ -1193,7 +1193,7 @@
     <t>TC144 Molina Cascade Bronze Zero WA-2027</t>
   </si>
   <si>
-    <t>Molina Cascade Bronze Zero</t>
+    <t>Schedule of Benefits – Molina Cascade Bronze Zero</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/english/WA27SOBE_B6_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/spanish/WA27SOBS_B6_2.pdf</t>
@@ -1202,7 +1202,7 @@
     <t>TC145 Molina Cascade Bronze LCS WA-2027</t>
   </si>
   <si>
-    <t>Molina Cascade Bronze LCS</t>
+    <t>Schedule of Benefits – Molina Cascade Bronze LCS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/english/WA27SOBE_B6_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/spanish/WA27SOBS_B6_3.pdf</t>
@@ -1211,7 +1211,7 @@
     <t>TC146 Molina Cascade Vital Gold WA-2027</t>
   </si>
   <si>
-    <t>Molina Cascade Vital Gold</t>
+    <t>Schedule of Benefits – Molina Cascade Vital Gold</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/english/WA27SOBE_G7_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/spanish/WA27SOBS_G7_1.pdf</t>
@@ -1220,7 +1220,7 @@
     <t>TC147 Molina Cascade Vital Gold Zero WA-2027</t>
   </si>
   <si>
-    <t>Molina Cascade Vital Gold Zero</t>
+    <t>Schedule of Benefits – Molina Cascade Vital Gold Zero</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/english/WA27SOBE_G7_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/spanish/WA27SOBS_G7_2.pdf</t>
@@ -1229,7 +1229,7 @@
     <t>TC148 Molina Cascade Vital Gold LCS WA-2027</t>
   </si>
   <si>
-    <t>Molina Cascade Vital Gold LCS</t>
+    <t>Schedule of Benefits – Molina Cascade Vital Gold LCS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/english/WA27SOBE_G7_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/wa/materials/SOB/2027/spanish/WA27SOBS_G7_3.pdf</t>
@@ -1241,7 +1241,7 @@
     <t>NM</t>
   </si>
   <si>
-    <t>Molina Gold Saver On Exchange</t>
+    <t>Schedule of Benefits – Molina Gold Saver On Exchange</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_G1_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_G1_1.pdf</t>
@@ -1250,7 +1250,7 @@
     <t>TC150 Molina Native American Gold Saver Zero NM-2027</t>
   </si>
   <si>
-    <t>Molina Native American Gold Saver Zero</t>
+    <t>Schedule of Benefits – Molina Native American Gold Saver Zero</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_G1_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_G1_2.pdf</t>
@@ -1259,7 +1259,7 @@
     <t>TC151 Molina Native American Gold Saver LCS NM-2027</t>
   </si>
   <si>
-    <t>Molina Native American Gold Saver LCS</t>
+    <t>Schedule of Benefits – Molina Native American Gold Saver LCS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_G1_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_G1_3.pdf</t>
@@ -1268,7 +1268,7 @@
     <t>TC152 Molina Native American Gold Saver Turquoise 3 LCS EXTRA SAVINGS NM-2027</t>
   </si>
   <si>
-    <t>Molina Native American Gold Saver Turquoise 3 LCS EXTRA SAVINGS</t>
+    <t>Schedule of Benefits – Molina Native American Gold Saver Turquoise 3 LCS EXTRA SAVINGS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_G1_13.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_G1_13.pdf</t>
@@ -1277,7 +1277,7 @@
     <t>TC153 Molina Gold Saver Turquoise 3 EXTRA SAVINGS NM-2027</t>
   </si>
   <si>
-    <t>Molina Gold Saver Turquoise 3 EXTRA SAVINGS</t>
+    <t>Schedule of Benefits – Molina Gold Saver Turquoise 3 EXTRA SAVINGS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_G1_90.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_G1_90.pdf</t>
@@ -1286,7 +1286,7 @@
     <t>TC154 Molina Clear Cost Gold On Exchange NM-2027</t>
   </si>
   <si>
-    <t>Molina Clear Cost Gold On Exchange</t>
+    <t>Schedule of Benefits – Molina Clear Cost Gold On Exchange</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_G13_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_G13_1.pdf</t>
@@ -1295,7 +1295,7 @@
     <t>TC155 Molina Native American Clear Cost Gold Zero NM-2027</t>
   </si>
   <si>
-    <t>Molina Native American Clear Cost Gold Zero</t>
+    <t>Schedule of Benefits – Molina Native American Clear Cost Gold Zero</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_G13_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_G13_2.pdf</t>
@@ -1304,7 +1304,7 @@
     <t>TC156 Molina Native American Clear Cost Gold LCS NM-2027</t>
   </si>
   <si>
-    <t>Molina Native American Clear Cost Gold LCS</t>
+    <t>Schedule of Benefits – Molina Native American Clear Cost Gold LCS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_G13_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_G13_3.pdf</t>
@@ -1313,7 +1313,7 @@
     <t>TC157 Molina Native American Clear Cost Turquoise 3 LCS EXTRA SAVINGS NM-2027</t>
   </si>
   <si>
-    <t>Molina Native American Clear Cost Turquoise 3 LCS EXTRA SAVINGS</t>
+    <t>Schedule of Benefits – Molina Native American Clear Cost Turquoise 3 LCS EXTRA SAVINGS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_G13_13.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_G13_13.pdf</t>
@@ -1322,7 +1322,7 @@
     <t>TC158 Molina Clear Cost Turquoise 3 EXTRA SAVINGS NM-2027</t>
   </si>
   <si>
-    <t>Molina Clear Cost Turquoise 3 EXTRA SAVINGS</t>
+    <t>Schedule of Benefits – Molina Clear Cost Turquoise 3 EXTRA SAVINGS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_G13_90.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_G13_90.pdf</t>
@@ -1331,7 +1331,7 @@
     <t>TC159 Molina Clear Cost Silver On Exchange NM-2027</t>
   </si>
   <si>
-    <t>Molina Clear Cost Silver On Exchange</t>
+    <t>Schedule of Benefits – Molina Clear Cost Silver On Exchange</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_S13_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_S13_1.pdf</t>
@@ -1340,7 +1340,7 @@
     <t>TC160 Molina Native American Clear Cost Silver Zero NM-2027</t>
   </si>
   <si>
-    <t>Molina Native American Clear Cost Silver Zero</t>
+    <t>Schedule of Benefits – Molina Native American Clear Cost Silver Zero</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_S13_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_S13_2.pdf</t>
@@ -1349,7 +1349,7 @@
     <t>TC161 Molina Native American Clear Cost Silver LCS NM-2027</t>
   </si>
   <si>
-    <t>Molina Native American Clear Cost Silver LCS</t>
+    <t>Schedule of Benefits – Molina Native American Clear Cost Silver LCS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_S13_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_S13_3.pdf</t>
@@ -1358,7 +1358,7 @@
     <t>TC162 Molina Clear Cost Silver 73 NM-2027</t>
   </si>
   <si>
-    <t>Molina Clear Cost Silver 73</t>
+    <t>Schedule of Benefits – Molina Clear Cost Silver 73</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_S13_4.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_S13_4.pdf</t>
@@ -1367,7 +1367,7 @@
     <t>TC163 Molina Clear Cost Silver 87 NM-2027</t>
   </si>
   <si>
-    <t>Molina Clear Cost Silver 87</t>
+    <t>Schedule of Benefits – Molina Clear Cost Silver 87</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_S13_9.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_S13_9.pdf</t>
@@ -1376,7 +1376,7 @@
     <t>TC164 Molina Clear Cost Silver 94 NM-2027</t>
   </si>
   <si>
-    <t>Molina Clear Cost Silver 94</t>
+    <t>Schedule of Benefits – Molina Clear Cost Silver 94</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_S13_5.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_S13_5.pdf</t>
@@ -1385,7 +1385,7 @@
     <t>TC165 Molina Clear Cost Turquoise 2 with EXTRA SAVINGS NM-2027</t>
   </si>
   <si>
-    <t>Molina Clear Cost Turquoise 2 with EXTRA SAVINGS</t>
+    <t>Schedule of Benefits – Molina Clear Cost Turquoise 2 with EXTRA SAVINGS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM26SOBE_S13_95.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM26SOBS_S13_95.pdf</t>
@@ -1394,7 +1394,7 @@
     <t>TC166 Molina Clear Cost Turquoise 1 with EXTRA SAVINGS NM-2027</t>
   </si>
   <si>
-    <t>Molina Clear Cost Turquoise 1 with EXTRA SAVINGS</t>
+    <t>Schedule of Benefits – Molina Clear Cost Turquoise 1 with EXTRA SAVINGS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM26SOBE_S13_99.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM26SOBS_S13_99.pdf</t>
@@ -1403,7 +1403,7 @@
     <t>TC167 Molina Silver Saver On Exchange NM-2027</t>
   </si>
   <si>
-    <t>Molina Silver Saver On Exchange</t>
+    <t>Schedule of Benefits – Molina Silver Saver On Exchange</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_S14_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_S14_1.pdf</t>
@@ -1412,7 +1412,7 @@
     <t>TC168 Molina Native American Silver Saver Zero NM-2027</t>
   </si>
   <si>
-    <t>Molina Native American Silver Saver Zero</t>
+    <t>Schedule of Benefits – Molina Native American Silver Saver Zero</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_S14_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_S14_2.pdf</t>
@@ -1421,7 +1421,7 @@
     <t>TC169 Molina Native American Silver Saver LCS NM-2027</t>
   </si>
   <si>
-    <t>Molina Native American Silver Saver LCS</t>
+    <t>Schedule of Benefits – Molina Native American Silver Saver LCS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_S14_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_S14_3.pdf</t>
@@ -1430,7 +1430,7 @@
     <t>TC170 Molina Silver Saver 73 NM-2027</t>
   </si>
   <si>
-    <t>Molina Silver Saver 73</t>
+    <t>Schedule of Benefits – Molina Silver Saver 73</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_S14_4.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_S14_4.pdf</t>
@@ -1439,7 +1439,7 @@
     <t>TC171 Molina Silver Saver 87 NM-2027</t>
   </si>
   <si>
-    <t>Molina Silver Saver 87</t>
+    <t>Schedule of Benefits – Molina Silver Saver 87</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_S14_9.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_S14_9.pdf</t>
@@ -1448,7 +1448,7 @@
     <t>TC172 Molina Silver Saver 94 NM-2027</t>
   </si>
   <si>
-    <t>Molina Silver Saver 94</t>
+    <t>Schedule of Benefits – Molina Silver Saver 94</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_S14_5.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_S14_5.pdf</t>
@@ -1457,7 +1457,7 @@
     <t>TC173 Molina Silver Saver Turquoise 2 with EXTRA SAVINGS NM-2027</t>
   </si>
   <si>
-    <t>Molina Silver Saver Turquoise 2 with EXTRA SAVINGS</t>
+    <t>Schedule of Benefits – Molina Silver Saver Turquoise 2 with EXTRA SAVINGS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM26SOBE_S14_95.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM26SOBS_S14_95.pdf</t>
@@ -1466,7 +1466,7 @@
     <t>TC174 Molina Silver Saver Turquoise 1 with EXTRA SAVINGS NM-2027</t>
   </si>
   <si>
-    <t>Molina Silver Saver Turquoise 1 with EXTRA SAVINGS</t>
+    <t>Schedule of Benefits – Molina Silver Saver Turquoise 1 with EXTRA SAVINGS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM26SOBE_S14_99.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM26SOBS_S14_99.pdf</t>
@@ -1475,7 +1475,7 @@
     <t>TC175 Molina Bronze Saver 7000 On Exchange NM-2027</t>
   </si>
   <si>
-    <t>Molina Bronze Saver 7000 On Exchange</t>
+    <t>Schedule of Benefits – Molina Bronze Saver 7000 On Exchange</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/english/NM27SOBE_B12_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nm/materials/SOB/2027/spanish/NM27SOBS_B12_1.pdf</t>
@@ -1499,7 +1499,7 @@
     <t>IL</t>
   </si>
   <si>
-    <t>Molina Open Gold Enhanced 750</t>
+    <t>Schedule of Benefits – Molina Open Gold Enhanced 750</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_G12_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_G12_1.pdf</t>
@@ -1508,7 +1508,7 @@
     <t>TC179 Molina Open Gold Enhanced Zero IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Gold Enhanced Zero</t>
+    <t>Schedule of Benefits – Molina Open Gold Enhanced Zero</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_G12_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_G12_2.pdf</t>
@@ -1517,7 +1517,7 @@
     <t>TC180 Molina Open Gold Enhanced 750 LCS IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Gold Enhanced 750 LCS</t>
+    <t>Schedule of Benefits – Molina Open Gold Enhanced 750 LCS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_G12_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_G12_3.pdf</t>
@@ -1526,7 +1526,7 @@
     <t>TC181 Molina Open Silver Empower 2750 IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Empower 2750</t>
+    <t>Schedule of Benefits – Molina Open Silver Empower 2750</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S16_0.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBS_S16_0.pdf</t>
@@ -1535,7 +1535,7 @@
     <t>TC182 Molina Open Silver Empower 4500 IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Empower 4500</t>
+    <t>Schedule of Benefits – Molina Open Silver Empower 4500</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S18_0.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBS_S18_0.pdf</t>
@@ -1544,7 +1544,7 @@
     <t>TC183 Molina Open Silver Empower 5500 IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Empower 5500</t>
+    <t>Schedule of Benefits – Molina Open Silver Empower 5500</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S19_0.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBS_S19_0.pdf</t>
@@ -1553,7 +1553,7 @@
     <t>TC184 Molina Open Gold Empower 2000 IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Gold Empower 2000</t>
+    <t>Schedule of Benefits – Molina Open Gold Empower 2000</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_G16_0.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBS_G16_0.pdf</t>
@@ -1562,7 +1562,7 @@
     <t>TC185 Molina Open Gold Empower 2000 Plus with Adult Vision IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Gold Empower 2000 Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Open Gold Empower 2000 Plus with Adult Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_G16V_0.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBS_G16V_0.pdf</t>
@@ -1571,7 +1571,7 @@
     <t>TC186 Molina Open Silver Empower 3750 Plus with Adult Dental and Vision IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Empower 3750 Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Open Silver Empower 3750 Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S17DV_0.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBS_S17DV_0.pdf</t>
@@ -1580,7 +1580,7 @@
     <t>TC187 Molina Open Gold Empower 2000 Plus with Adult Dental and Vision IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Gold Empower 2000 Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Open Gold Empower 2000 Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_G16DV_0.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBS_G16DV_0.pdf</t>
@@ -1589,7 +1589,7 @@
     <t>TC188 Molina Open Gold Core 1500 IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Gold Core 1500</t>
+    <t>Schedule of Benefits – Molina Open Gold Core 1500</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_G1_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_G1_1.pdf</t>
@@ -1598,7 +1598,7 @@
     <t>TC189 Molina Open Gold Core Zero IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Gold Core Zero</t>
+    <t>Schedule of Benefits – Molina Open Gold Core Zero</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_G1_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_G1_2.pdf</t>
@@ -1607,7 +1607,7 @@
     <t>TC190 Molina Open Gold Core 1500 LCS IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Gold Core 1500 LCS</t>
+    <t>Schedule of Benefits – Molina Open Gold Core 1500 LCS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_G1_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_G1_3.pdf</t>
@@ -1616,7 +1616,7 @@
     <t>TC191 Molina Open Silver Core 70 IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Core 70</t>
+    <t>Schedule of Benefits – Molina Open Silver Core 70</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S1_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S1_1.pdf</t>
@@ -1625,7 +1625,7 @@
     <t>TC192 Molina Open Silver Core Zero IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Core Zero</t>
+    <t>Schedule of Benefits – Molina Open Silver Core Zero</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S1_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S1_2.pdf</t>
@@ -1634,7 +1634,7 @@
     <t>TC193 Molina Open Silver Core 70 LCS IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Core 70 LCS</t>
+    <t>Schedule of Benefits – Molina Open Silver Core 70 LCS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S1_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S1_3.pdf</t>
@@ -1643,7 +1643,7 @@
     <t>TC194 Molina Open Silver Core 73 IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Core 73</t>
+    <t>Schedule of Benefits – Molina Open Silver Core 73</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S1_4.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S1_4.pdf</t>
@@ -1652,7 +1652,7 @@
     <t>TC195 Molina Open Silver Core 87 IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Core 87</t>
+    <t>Schedule of Benefits – Molina Open Silver Core 87</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S1_5.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S1_5.pdf</t>
@@ -1661,7 +1661,7 @@
     <t>TC196 Molina Open Silver Core 94 IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Core 94</t>
+    <t>Schedule of Benefits – Molina Open Silver Core 94</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S1_6.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S1_6.pdf</t>
@@ -1670,7 +1670,7 @@
     <t>TC197 Molina Open Silver Saver 70 with Four Free PCP or MH Visits IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Saver 70 with Four Free PCP or MH Visits</t>
+    <t>Schedule of Benefits – Molina Open Silver Saver 70 with Four Free PCP or MH Visits</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S12_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S12_1.pdf</t>
@@ -1679,7 +1679,7 @@
     <t>TC198 Molina Open Silver Saver Zero IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Saver Zero</t>
+    <t>Schedule of Benefits – Molina Open Silver Saver Zero</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S12_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S12_2.pdf</t>
@@ -1688,7 +1688,7 @@
     <t>TC199 Molina Open Silver Saver  LCS with Four Free PCP or MH Visits IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Saver  LCS with Four Free PCP or MH Visits</t>
+    <t>Schedule of Benefits – Molina Open Silver Saver  LCS with Four Free PCP or MH Visits</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S12_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S12_3.pdf</t>
@@ -1697,7 +1697,7 @@
     <t>TC200 Molina Open Silver Saver 73 with Four Free PCP or MH Visits IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Saver 73 with Four Free PCP or MH Visits</t>
+    <t>Schedule of Benefits – Molina Open Silver Saver 73 with Four Free PCP or MH Visits</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S12_4.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S12_4.pdf</t>
@@ -1706,7 +1706,7 @@
     <t>TC201 Molina Open Silver Saver 87 with Four Free PCP or MH Visits IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Saver 87 with Four Free PCP or MH Visits</t>
+    <t>Schedule of Benefits – Molina Open Silver Saver 87 with Four Free PCP or MH Visits</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S12_5.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S12_5.pdf</t>
@@ -1715,7 +1715,7 @@
     <t>TC202 Molina Open Silver Saver 94 with Four Free PCP or MH Visits IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Saver 94 with Four Free PCP or MH Visits</t>
+    <t>Schedule of Benefits – Molina Open Silver Saver 94 with Four Free PCP or MH Visits</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S12_6.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S12_6.pdf</t>
@@ -1724,7 +1724,7 @@
     <t>TC203 Molina Open Gold Core 1500 Plus with Adult Vision IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Gold Core 1500 Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Open Gold Core 1500 Plus with Adult Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_G1V_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_G1V_1.pdf</t>
@@ -1733,7 +1733,7 @@
     <t>TC204 Molina Open Gold Core Zero Plus with Adult Vision IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Gold Core Zero Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Open Gold Core Zero Plus with Adult Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_G1V_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_G1V_2.pdf</t>
@@ -1742,7 +1742,7 @@
     <t>TC205 Molina Open Gold Core 1500 LCS Plus with Adult Vision IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Gold Core 1500 LCS Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Open Gold Core 1500 LCS Plus with Adult Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_G1V_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_G1V_3.pdf</t>
@@ -1751,7 +1751,7 @@
     <t>TC206 Molina Open Silver Core 70 Plus with Adult Vision IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Core 70 Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Open Silver Core 70 Plus with Adult Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S1V_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S1V_1.pdf</t>
@@ -1760,7 +1760,7 @@
     <t>TC207 Molina Open Silver Core Zero Plus with Adult Vision IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Core Zero Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Open Silver Core Zero Plus with Adult Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S1V_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S1V_2.pdf</t>
@@ -1769,7 +1769,7 @@
     <t>TC208 Molina Open Silver Core 70 LCS Plus with Adult Vision IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Core 70 LCS Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Open Silver Core 70 LCS Plus with Adult Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S1V_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S1V_3.pdf</t>
@@ -1778,7 +1778,7 @@
     <t>TC209 Molina Open Silver Core 73 Plus with Adult Vision IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Core 73 Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Open Silver Core 73 Plus with Adult Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S1V_4.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S1V_4.pdf</t>
@@ -1787,7 +1787,7 @@
     <t>TC210 Molina Open Silver Core 87 Plus with Adult Vision IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Core 87 Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Open Silver Core 87 Plus with Adult Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S1V_5.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S1V_5.pdf</t>
@@ -1796,7 +1796,7 @@
     <t>TC211 Molina Open Silver Core 94 Plus with Adult Vision IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Core 94 Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Open Silver Core 94 Plus with Adult Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S1V_6.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S1V_6.pdf</t>
@@ -1805,7 +1805,7 @@
     <t>TC212 Molina Open Gold Core 1500 Plus with Rx Copay and Adult Dental and Vision IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Gold Core 1500 Plus with Rx Copay and Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Open Gold Core 1500 Plus with Rx Copay and Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_G1DV_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_G1DV_1.pdf</t>
@@ -1814,7 +1814,7 @@
     <t>TC213 Molina Open Gold Core Zero Plus with Rx Copay and Adult Dental and Vision IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Gold Core Zero Plus with Rx Copay and Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Open Gold Core Zero Plus with Rx Copay and Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_G1DV_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_G1DV_2.pdf</t>
@@ -1823,7 +1823,7 @@
     <t>TC214 Molina Open Gold Core 1500 LCS Plus with Rx Copay and Adult Dental and Vision IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Gold Core 1500 LCS Plus with Rx Copay and Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Open Gold Core 1500 LCS Plus with Rx Copay and Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_G1DV_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_G1DV_3.pdf</t>
@@ -1832,7 +1832,7 @@
     <t>TC215 Molina Open Silver Core 70 Plus with Rx Copay and Adult Dental and Vision IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Core 70 Plus with Rx Copay and Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Open Silver Core 70 Plus with Rx Copay and Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S1DV_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S1DV_1.pdf</t>
@@ -1841,7 +1841,7 @@
     <t>TC216 Molina Open Silver Core Zero Plus with Rx Copay and Adult Dental and Vision IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Core Zero Plus with Rx Copay and Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Open Silver Core Zero Plus with Rx Copay and Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S1DV_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S1DV_2.pdf</t>
@@ -1856,7 +1856,7 @@
     <t>TC218 Molina Open Silver Core 73 Plus with Rx Copay and Adult Dental and Vision IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Core 73 Plus with Rx Copay and Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Open Silver Core 73 Plus with Rx Copay and Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S1DV_4.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S1DV_4.pdf</t>
@@ -1865,7 +1865,7 @@
     <t>TC219 Molina Open Silver Core 87 Plus with Rx Copay and Adult Dental and Vision IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Core 87 Plus with Rx Copay and Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Open Silver Core 87 Plus with Rx Copay and Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S1DV_5.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S1DV_5.pdf</t>
@@ -1874,7 +1874,7 @@
     <t>TC220 Molina Open Silver Core 94 Plus with Rx Copay and Adult Dental and Vision IL-2027</t>
   </si>
   <si>
-    <t>Molina Open Silver Core 94 Plus with Rx Copay and Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Open Silver Core 94 Plus with Rx Copay and Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/english/IL27SOBE_S1DV_6.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/il/materials/SOB/2027/spanish/IL27SOBS_S1DV_6.pdf</t>
@@ -2030,7 +2030,7 @@
     <t>TC245 Molina Gold Enhanced 750 Plus with Adult Dental and Vision MI-2027</t>
   </si>
   <si>
-    <t>Molina Gold Enhanced 750 Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Gold Enhanced 750 Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/mi/materials/SOB/2027/english/MI27SOBE_G12DV_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/mi/materials/SOB/2027/spanish/MI27SOBS_G12DV_1.pdf</t>
@@ -2045,7 +2045,7 @@
     <t>TC247 Molina Gold Enhanced 750 LCS Plus with Adult Dental and Vision MI-2027</t>
   </si>
   <si>
-    <t>Molina Gold Enhanced 750 LCS Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Gold Enhanced 750 LCS Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/mi/materials/SOB/2027/english/MI27SOBE_G12DV_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/mi/materials/SOB/2027/spanish/MI27SOBS_G12DV_3.pdf</t>
@@ -2057,7 +2057,7 @@
     <t>TX</t>
   </si>
   <si>
-    <t>Silver 3</t>
+    <t>Schedule of Benefits – Silver 3</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/SOB/2027/english/TX27SOBE_S3_0.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/SOB/2027/spanish/TX27SOBS_S3_0.pdf</t>
@@ -2156,7 +2156,7 @@
     <t>TC264 Molina Gold Enhanced 750 TX-2027</t>
   </si>
   <si>
-    <t>Molina Gold Enhanced 750</t>
+    <t>Schedule of Benefits – Molina Gold Enhanced 750</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/SOB/2027/english/TX27SOBE_G12_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/SOB/2027/spanish/TX27SOBS_G12_1.pdf</t>
@@ -2171,7 +2171,7 @@
     <t>TC266 Molina Gold Enhanced 750 LCS TX-2027</t>
   </si>
   <si>
-    <t>Molina Gold Enhanced 750 LCS</t>
+    <t>Schedule of Benefits – Molina Gold Enhanced 750 LCS</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/SOB/2027/english/TX27SOBE_G12_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/SOB/2027/spanish/TX27SOBS_G12_3.pdf</t>
@@ -2264,7 +2264,7 @@
     <t>TC281 Molina Gold Saver 750 Plus with Adult Vision TX-2027</t>
   </si>
   <si>
-    <t>Molina Gold Saver 750 Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Gold Saver 750 Plus with Adult Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/SOB/2027/english/TX27SOBE_G12V_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/SOB/2027/spanish/TX27SOBS_G12V_1.pdf</t>
@@ -2273,7 +2273,7 @@
     <t>TC282 Molina Gold Saver Zero Plus with Adult Vision TX-2027</t>
   </si>
   <si>
-    <t>Molina Gold Saver Zero Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Gold Saver Zero Plus with Adult Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/SOB/2027/english/TX27SOBE_G12V_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/SOB/2027/spanish/TX27SOBS_G12V_2.pdf</t>
@@ -2282,7 +2282,7 @@
     <t>TC283 Molina Gold Saver 750 LCS Plus with Adult Vision TX-2027</t>
   </si>
   <si>
-    <t>Molina Gold Saver 750 LCS Plus with Adult Vision</t>
+    <t>Schedule of Benefits – Molina Gold Saver 750 LCS Plus with Adult Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/SOB/2027/english/TX27SOBE_G12V_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/SOB/2027/spanish/TX27SOBS_G12V_3.pdf</t>
@@ -2351,7 +2351,7 @@
     <t>TC294 Molina Silver Core 70 LCS Plus with Adult Dental and Vision TX-2027</t>
   </si>
   <si>
-    <t>Molina Silver Core 70 LCS Plus with Adult Dental and Vision</t>
+    <t>Schedule of Benefits – Molina Silver Core 70 LCS Plus with Adult Dental and Vision</t>
   </si>
   <si>
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/SOB/2027/english/TX27SOBE_S1DV_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/SOB/2027/spanish/TX27SOBS_S1DV_3.pdf</t>
@@ -2423,82 +2423,82 @@
     <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/SOB/2027/english/TX27SOBE_G16DV_0.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/tx/materials/SOB/2027/spanish/TX27SOBS_G16DV_0.pdf</t>
   </si>
   <si>
+    <t>TC306 Molina Gold Core 1500 Plus with Adult Vision NV-2027</t>
+  </si>
+  <si>
+    <t>NV</t>
+  </si>
+  <si>
+    <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/english/NV27SOBE_G1V_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/spanish/NV27SOBS_G1V_1.pdf</t>
+  </si>
+  <si>
+    <t>TC307 Molina Gold Core Zero Plus with Adult Vision NV-2027</t>
+  </si>
+  <si>
+    <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/english/NV27SOBE_G1V_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/spanish/NV27SOBS_G1V_2.pdf</t>
+  </si>
+  <si>
+    <t>TC308 Molina Gold Core 1500 LCS Plus with Adult Vision NV-2027</t>
+  </si>
+  <si>
+    <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/english/NV27SOBE_G1V_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/spanish/NV27SOBS_G1V_3.pdf</t>
+  </si>
+  <si>
+    <t>TC309 Molina Silver Core 70 Plus with Adult Vision NV-2027</t>
+  </si>
+  <si>
+    <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/english/NV27SOBE_S1V_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/spanish/NV27SOBS_S1V_1.pdf</t>
+  </si>
+  <si>
+    <t>TC310 Molina Silver Core Zero Plus with Adult Vision NV-2027</t>
+  </si>
+  <si>
+    <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/english/NV27SOBE_S1V_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/spanish/NV27SOBS_S1V_2.pdf</t>
+  </si>
+  <si>
+    <t>TC311 Molina Silver Core LCS Plus with Adult Vision NV-2027</t>
+  </si>
+  <si>
+    <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/english/NV27SOBE_S1V_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/spanish/NV27SOBS_S1V_3.pdf</t>
+  </si>
+  <si>
+    <t>TC312 Molina Silver Core 73 Plus with Adult Vision NV-2027</t>
+  </si>
+  <si>
+    <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/english/NV27SOBE_S1V_4.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/spanish/NV27SOBS_S1V_4.pdf</t>
+  </si>
+  <si>
+    <t>TC313 Molina Silver Core 87 Plus with Adult Vision NV-2027</t>
+  </si>
+  <si>
+    <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/english/NV27SOBE_S1V_5.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/spanish/NV27SOBS_S1V_5.pdf</t>
+  </si>
+  <si>
+    <t>TC314 Molina Silver Core 94 Plus with Adult Vision NV-2027</t>
+  </si>
+  <si>
+    <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/english/NV27SOBE_S1V_6.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/spanish/NV27SOBS_S1V_6.pdf</t>
+  </si>
+  <si>
+    <t>Key</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>AppUrl</t>
+  </si>
+  <si>
+    <t>https://uat-pws.molinahealthcare.com/</t>
+  </si>
+  <si>
+    <t>Landing URL for the Plan Search suite. Change to point at Q1/Q2/Q3/UAT/prod without editing code. Precedence: MARKETPLACE_PLANS_URL env var &gt; this Value &gt; framework.config.js default.</t>
+  </si>
+  <si>
     <t>Y</t>
-  </si>
-  <si>
-    <t>TC306 Molina Gold Core 1500 Plus with Adult Vision NV-2027</t>
-  </si>
-  <si>
-    <t>NV</t>
-  </si>
-  <si>
-    <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/english/NV27SOBE_G1V_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/spanish/NV27SOBS_G1V_1.pdf</t>
-  </si>
-  <si>
-    <t>TC307 Molina Gold Core Zero Plus with Adult Vision NV-2027</t>
-  </si>
-  <si>
-    <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/english/NV27SOBE_G1V_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/spanish/NV27SOBS_G1V_2.pdf</t>
-  </si>
-  <si>
-    <t>TC308 Molina Gold Core 1500 LCS Plus with Adult Vision NV-2027</t>
-  </si>
-  <si>
-    <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/english/NV27SOBE_G1V_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/spanish/NV27SOBS_G1V_3.pdf</t>
-  </si>
-  <si>
-    <t>TC309 Molina Silver Core 70 Plus with Adult Vision NV-2027</t>
-  </si>
-  <si>
-    <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/english/NV27SOBE_S1V_1.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/spanish/NV27SOBS_S1V_1.pdf</t>
-  </si>
-  <si>
-    <t>TC310 Molina Silver Core Zero Plus with Adult Vision NV-2027</t>
-  </si>
-  <si>
-    <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/english/NV27SOBE_S1V_2.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/spanish/NV27SOBS_S1V_2.pdf</t>
-  </si>
-  <si>
-    <t>TC311 Molina Silver Core LCS Plus with Adult Vision NV-2027</t>
-  </si>
-  <si>
-    <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/english/NV27SOBE_S1V_3.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/spanish/NV27SOBS_S1V_3.pdf</t>
-  </si>
-  <si>
-    <t>TC312 Molina Silver Core 73 Plus with Adult Vision NV-2027</t>
-  </si>
-  <si>
-    <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/english/NV27SOBE_S1V_4.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/spanish/NV27SOBS_S1V_4.pdf</t>
-  </si>
-  <si>
-    <t>TC313 Molina Silver Core 87 Plus with Adult Vision NV-2027</t>
-  </si>
-  <si>
-    <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/english/NV27SOBE_S1V_5.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/spanish/NV27SOBS_S1V_5.pdf</t>
-  </si>
-  <si>
-    <t>TC314 Molina Silver Core 94 Plus with Adult Vision NV-2027</t>
-  </si>
-  <si>
-    <t>https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/english/NV27SOBE_S1V_6.pdf|https://www.molinahealthcare.com/-/media/project/pws/healthcare/pdf/pdf/ifp/nv/materials/SOB/2027/spanish/NV27SOBS_S1V_6.pdf</t>
-  </si>
-  <si>
-    <t>Key</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>AppUrl</t>
-  </si>
-  <si>
-    <t>https://uat-pws.molinahealthcare.com/</t>
-  </si>
-  <si>
-    <t>Landing URL for the Plan Search suite. Change to point at Q1/Q2/Q3/UAT/prod without editing code. Precedence: MARKETPLACE_PLANS_URL env var &gt; this Value &gt; framework.config.js default.</t>
   </si>
 </sst>
 </file>
@@ -2599,10 +2599,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -2634,10 +2634,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -2879,10 +2879,10 @@
   <dimension ref="A1:I315"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="6" max="6" width="11.296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.09765625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="70.3984375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="241.19921875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.296875" customWidth="1"/>
+    <col min="7" max="7" width="18.09765625" customWidth="1"/>
+    <col min="8" max="8" width="70.3984375" customWidth="1"/>
+    <col min="9" max="9" width="241.19921875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
@@ -5437,9 +5437,9 @@
         <v>260</v>
       </c>
     </row>
-    <row r="89" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B89" t="s">
         <v>261</v>
@@ -5466,9 +5466,9 @@
         <v>263</v>
       </c>
     </row>
-    <row r="90" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B90" t="s">
         <v>264</v>
@@ -5495,9 +5495,9 @@
         <v>265</v>
       </c>
     </row>
-    <row r="91" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B91" t="s">
         <v>266</v>
@@ -5524,9 +5524,9 @@
         <v>267</v>
       </c>
     </row>
-    <row r="92" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B92" t="s">
         <v>268</v>
@@ -5553,9 +5553,9 @@
         <v>269</v>
       </c>
     </row>
-    <row r="93" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B93" t="s">
         <v>270</v>
@@ -5582,9 +5582,9 @@
         <v>271</v>
       </c>
     </row>
-    <row r="94" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B94" t="s">
         <v>272</v>
@@ -5611,9 +5611,9 @@
         <v>273</v>
       </c>
     </row>
-    <row r="95" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B95" t="s">
         <v>274</v>
@@ -5640,9 +5640,9 @@
         <v>275</v>
       </c>
     </row>
-    <row r="96" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B96" t="s">
         <v>276</v>
@@ -5669,9 +5669,9 @@
         <v>277</v>
       </c>
     </row>
-    <row r="97" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B97" t="s">
         <v>278</v>
@@ -5698,9 +5698,9 @@
         <v>279</v>
       </c>
     </row>
-    <row r="98" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B98" t="s">
         <v>280</v>
@@ -5727,9 +5727,9 @@
         <v>281</v>
       </c>
     </row>
-    <row r="99" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B99" t="s">
         <v>282</v>
@@ -5756,9 +5756,9 @@
         <v>283</v>
       </c>
     </row>
-    <row r="100" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B100" t="s">
         <v>284</v>
@@ -5785,9 +5785,9 @@
         <v>285</v>
       </c>
     </row>
-    <row r="101" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B101" t="s">
         <v>286</v>
@@ -5814,9 +5814,9 @@
         <v>287</v>
       </c>
     </row>
-    <row r="102" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B102" t="s">
         <v>288</v>
@@ -5843,9 +5843,9 @@
         <v>289</v>
       </c>
     </row>
-    <row r="103" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B103" t="s">
         <v>290</v>
@@ -5872,9 +5872,9 @@
         <v>291</v>
       </c>
     </row>
-    <row r="104" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B104" t="s">
         <v>292</v>
@@ -5901,9 +5901,9 @@
         <v>293</v>
       </c>
     </row>
-    <row r="105" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B105" t="s">
         <v>294</v>
@@ -5930,9 +5930,9 @@
         <v>295</v>
       </c>
     </row>
-    <row r="106" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B106" t="s">
         <v>296</v>
@@ -5959,9 +5959,9 @@
         <v>297</v>
       </c>
     </row>
-    <row r="107" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B107" t="s">
         <v>298</v>
@@ -5988,9 +5988,9 @@
         <v>299</v>
       </c>
     </row>
-    <row r="108" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B108" t="s">
         <v>300</v>
@@ -6017,9 +6017,9 @@
         <v>301</v>
       </c>
     </row>
-    <row r="109" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B109" t="s">
         <v>302</v>
@@ -6046,9 +6046,9 @@
         <v>303</v>
       </c>
     </row>
-    <row r="110" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B110" t="s">
         <v>304</v>
@@ -6075,9 +6075,9 @@
         <v>305</v>
       </c>
     </row>
-    <row r="111" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B111" t="s">
         <v>306</v>
@@ -6104,9 +6104,9 @@
         <v>307</v>
       </c>
     </row>
-    <row r="112" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B112" t="s">
         <v>308</v>
@@ -6133,9 +6133,9 @@
         <v>309</v>
       </c>
     </row>
-    <row r="113" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B113" t="s">
         <v>310</v>
@@ -6162,9 +6162,9 @@
         <v>311</v>
       </c>
     </row>
-    <row r="114" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B114" t="s">
         <v>312</v>
@@ -6191,9 +6191,9 @@
         <v>313</v>
       </c>
     </row>
-    <row r="115" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B115" t="s">
         <v>314</v>
@@ -6220,9 +6220,9 @@
         <v>315</v>
       </c>
     </row>
-    <row r="116" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B116" t="s">
         <v>316</v>
@@ -6249,9 +6249,9 @@
         <v>317</v>
       </c>
     </row>
-    <row r="117" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B117" t="s">
         <v>318</v>
@@ -6278,9 +6278,9 @@
         <v>319</v>
       </c>
     </row>
-    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B118" t="s">
         <v>320</v>
@@ -6307,9 +6307,9 @@
         <v>321</v>
       </c>
     </row>
-    <row r="119" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B119" t="s">
         <v>322</v>
@@ -6336,9 +6336,9 @@
         <v>323</v>
       </c>
     </row>
-    <row r="120" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B120" t="s">
         <v>324</v>
@@ -6365,9 +6365,9 @@
         <v>325</v>
       </c>
     </row>
-    <row r="121" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
-        <v>9</v>
+        <v>824</v>
       </c>
       <c r="B121" t="s">
         <v>326</v>
@@ -11759,15 +11759,15 @@
         <v>798</v>
       </c>
     </row>
-    <row r="307" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>9</v>
       </c>
       <c r="B307" t="s">
+        <v>799</v>
+      </c>
+      <c r="C307" t="s">
         <v>800</v>
-      </c>
-      <c r="C307" t="s">
-        <v>801</v>
       </c>
       <c r="D307" t="s">
         <v>12</v>
@@ -11785,18 +11785,18 @@
         <v>106</v>
       </c>
       <c r="I307" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="308" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A308" t="s">
+        <v>9</v>
+      </c>
+      <c r="B308" t="s">
         <v>802</v>
       </c>
-    </row>
-    <row r="308" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A308" t="s">
-        <v>9</v>
-      </c>
-      <c r="B308" t="s">
-        <v>803</v>
-      </c>
       <c r="C308" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="D308" t="s">
         <v>12</v>
@@ -11814,18 +11814,18 @@
         <v>109</v>
       </c>
       <c r="I308" t="s">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="309" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A309" t="s">
+        <v>9</v>
+      </c>
+      <c r="B309" t="s">
         <v>804</v>
       </c>
-    </row>
-    <row r="309" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A309" t="s">
-        <v>9</v>
-      </c>
-      <c r="B309" t="s">
-        <v>805</v>
-      </c>
       <c r="C309" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="D309" t="s">
         <v>12</v>
@@ -11843,18 +11843,18 @@
         <v>112</v>
       </c>
       <c r="I309" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="310" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A310" t="s">
+        <v>9</v>
+      </c>
+      <c r="B310" t="s">
         <v>806</v>
       </c>
-    </row>
-    <row r="310" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A310" t="s">
-        <v>9</v>
-      </c>
-      <c r="B310" t="s">
-        <v>807</v>
-      </c>
       <c r="C310" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="D310" t="s">
         <v>12</v>
@@ -11872,18 +11872,18 @@
         <v>115</v>
       </c>
       <c r="I310" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="311" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A311" t="s">
+        <v>9</v>
+      </c>
+      <c r="B311" t="s">
         <v>808</v>
       </c>
-    </row>
-    <row r="311" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A311" t="s">
-        <v>9</v>
-      </c>
-      <c r="B311" t="s">
-        <v>809</v>
-      </c>
       <c r="C311" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="D311" t="s">
         <v>12</v>
@@ -11901,18 +11901,18 @@
         <v>118</v>
       </c>
       <c r="I311" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="312" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A312" t="s">
+        <v>9</v>
+      </c>
+      <c r="B312" t="s">
         <v>810</v>
       </c>
-    </row>
-    <row r="312" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A312" t="s">
-        <v>799</v>
-      </c>
-      <c r="B312" t="s">
-        <v>811</v>
-      </c>
       <c r="C312" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="D312" t="s">
         <v>12</v>
@@ -11930,18 +11930,18 @@
         <v>121</v>
       </c>
       <c r="I312" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="313" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A313" t="s">
+        <v>9</v>
+      </c>
+      <c r="B313" t="s">
         <v>812</v>
       </c>
-    </row>
-    <row r="313" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A313" t="s">
-        <v>799</v>
-      </c>
-      <c r="B313" t="s">
-        <v>813</v>
-      </c>
       <c r="C313" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="D313" t="s">
         <v>12</v>
@@ -11959,18 +11959,18 @@
         <v>124</v>
       </c>
       <c r="I313" t="s">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="314" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A314" t="s">
+        <v>9</v>
+      </c>
+      <c r="B314" t="s">
         <v>814</v>
       </c>
-    </row>
-    <row r="314" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A314" t="s">
-        <v>9</v>
-      </c>
-      <c r="B314" t="s">
-        <v>815</v>
-      </c>
       <c r="C314" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="D314" t="s">
         <v>12</v>
@@ -11988,18 +11988,18 @@
         <v>127</v>
       </c>
       <c r="I314" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="315" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A315" t="s">
+        <v>9</v>
+      </c>
+      <c r="B315" t="s">
         <v>816</v>
       </c>
-    </row>
-    <row r="315" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A315" t="s">
-        <v>9</v>
-      </c>
-      <c r="B315" t="s">
-        <v>817</v>
-      </c>
       <c r="C315" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="D315" t="s">
         <v>12</v>
@@ -12017,20 +12017,20 @@
         <v>130</v>
       </c>
       <c r="I315" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I315" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="2">
       <filters>
-        <filter val="NV"/>
+        <filter val="ID"/>
       </filters>
     </filterColumn>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:I306 A312:I313 B307:I307 B308:I311 B315:I315 B314:I314" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:I2 B116:I315 B115:I115 B3:I114" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -12047,24 +12047,24 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>818</v>
+      </c>
+      <c r="B1" t="s">
         <v>819</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>820</v>
-      </c>
-      <c r="C1" t="s">
-        <v>821</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>821</v>
+      </c>
+      <c r="B2" t="s">
         <v>822</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>823</v>
-      </c>
-      <c r="C2" t="s">
-        <v>824</v>
       </c>
     </row>
   </sheetData>

</xml_diff>